<commit_message>
Daily job scan: 2026-08-21
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -493,51 +493,51 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COSTING ENGINEER</t>
+          <t>Backend Developer- Python</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Coimbatore South,</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>data (tag), engineer, coimbatore (place)</t>
+          <t>python, backend, developer, bangalore (place)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>customer support, marketing, exec, golang, data entry, infosec, finance, excel, full time, design, math, ops, engineer, digital nomad, sales, technical, dev, testing, education, assembly, ruby</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-costing-engineer-larsen-amp-toubro-1137012</t>
+          <t>https://www.adzuna.in/land/ad/5837138703?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=21D74D2D75ABF8D23E544DFE97E76A06BBA93975</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>cda3327e13</t>
+          <t>3c0cf7d04b</t>
         </is>
       </c>
     </row>
@@ -548,51 +548,51 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Junior Scrum Master</t>
+          <t>Junior Architect</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Vonage</t>
+          <t>Arete Design Studio</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>junior, anywhere (place)</t>
+          <t>junior, india (place), chandigarh (place)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>Creative &amp; Design Jobs</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/vonage-junior-scrum-master</t>
+          <t>https://www.adzuna.in/land/ad/5849577279?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=DCCAD052B37E93CB8A85F717F402A53B14889A34</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>9e2bd601cd</t>
+          <t>9fe581aa32</t>
         </is>
       </c>
     </row>
@@ -603,51 +603,51 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRC Analyst</t>
+          <t>Data Automation engineer, NCT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Deutsche Bank</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>analyst, anywhere (place)</t>
+          <t>data, automation, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Front-End Programming, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/vercel-grc-analyst</t>
+          <t>https://www.adzuna.in/land/ad/5847959661?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=3294EC7E7CD15763384B4A67E7F012AD1307ACCE</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>51606110dd</t>
+          <t>a9c8421191</t>
         </is>
       </c>
     </row>
@@ -658,51 +658,51 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Vice President Data Operations - Transformation &amp; Automation</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Coimbatore, Tamil Nadu</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>data, automation, coimbatore (place)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5785771397?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=9FB87F5D2ED64B39DBC4C8AF4F231B7D3664AE1D</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>8a8666d796</t>
         </is>
       </c>
     </row>
@@ -713,51 +713,51 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Automation Engineer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Dhruv Technology Solutions</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>engineer, anywhere (place)</t>
+          <t>automation, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Engineering Jobs</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5825071019?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=240A1CF93A011217AAF1F2D22ECD71BFB24210E7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>4898883b52</t>
         </is>
       </c>
     </row>
@@ -768,51 +768,51 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Precast Design Engineer</t>
+          <t>Automation Developer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fisher Associates, P.e., L.s., L.a., D.</t>
+          <t>WPP Production</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>engineer, anywhere (place)</t>
+          <t>automation, developer, hyderabad (place)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/fisher-associates-p-e-l-s-l-a-d-precast-design-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5785771269?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1DDE4440D25853CB5AC581E115C01B6AAF4DD064</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>35e1092dfa</t>
+          <t>505b347559</t>
         </is>
       </c>
     </row>
@@ -823,51 +823,51 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Customer Success Engineer</t>
+          <t>Automation Engineer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Noida, Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>engineer, anywhere (place)</t>
+          <t>automation, engineer, noida (place)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Customer Support, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/hightouch-customer-success-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139113?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4F2A638A617FCEA4FF5170EB9BC5F703C29EE807</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>7859de02e2</t>
+          <t>cb75f6ffb1</t>
         </is>
       </c>
     </row>
@@ -878,51 +878,51 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tier III Service Desk Engineer</t>
+          <t>Automation Engineer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unio Digital</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Noida, Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>remotive</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>engineer, worldwide (place)</t>
+          <t>automation, engineer, noida (place)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Information Technology, full_time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://remotive.com/remote-jobs/information-technology/tier-iii-service-desk-engineer-2091045</t>
+          <t>https://www.adzuna.in/land/ad/5837843504?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=3DC1B50ECB81D0C561386188E5944C4C581D3F9C</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>17f629b43a</t>
+          <t>168afe012d</t>
         </is>
       </c>
     </row>
@@ -933,49 +933,1974 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>26</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AI and Automation Developer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>automation, developer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>f805954e2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>26</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Automation QA Test Engineer</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>automation, engineer, pune (place)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5849297018?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CF35C9FED96943041B64EA3F35B9B5D509EFF332</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>78e5ec5e29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>26</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Automation Engineer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Kyndryl</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>automation, engineer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5837139069?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=273094A6E829428657022EC1461D85E1A2F7CCC5</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0f3d858482</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>26</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Junior Analyst - India</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>junior, analyst, pune (place)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance Jobs</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850906792?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7908288D458D5C545B91878A4CD513D07FE33259</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>3531d0a24c</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>23</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>COSTING ENGINEER</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Coimbatore South,</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>remoteok</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>data (tag), engineer, coimbatore (place)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>customer support, marketing, exec, golang, data entry, infosec, finance, excel, full time, design, math, ops, engineer, digital nomad, sales, technical, dev, testing, education, assembly, ruby</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-costing-engineer-larsen-amp-toubro-1137012</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>cda3327e13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>23</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>The Ministry Of Light</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Worli, Mumbai</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>junior, engineer (tag), mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Engineering Jobs</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5804795868?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=5086836B50D76429020F9F40D709C7C19401A301</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>6ced295af0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Backend Operations</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mastek</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>backend, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Admin Jobs</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5821438925?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=5AEEC7568FE6214D452CF83F6DE6B092DAFAD898</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>b8c84e0c6a</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>21</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pinacche Artificer</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>junior, delhi (place)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983494?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=9150D8558489604EF3C1EE46A08E767E598908AE</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>79f926b1d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>21</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Junior GIS Technician</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AgriCapture</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>junior, india (place)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Scientific &amp; QA Jobs</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983089?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=6DFAAF8B16C782B85407F5405B4F74B591DAD55C</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>aa82b1f59e</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>21</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Junior Accountant</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>RTC India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>junior, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance Jobs</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5847166681?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=559F5962BB27AF1426787B4813EFF766FD7A4AAD</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>bd813a6ba4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>21</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Junior Accountant</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Zemoso Technologies</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>junior, hyderabad (place)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance Jobs</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5819622820?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1DB181C545E89DD49ECAABD2D53E010067B59EFF</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>e82d9d4af1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>21</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Junior Accountant</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Raya Software Solutions</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>junior, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance Jobs</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5845683345?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=42E42947ECE52DB0AB62410FF00261CEB721315D</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>6035f8d7ac</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Junior Copywriter</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Adfactors PR</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>junior, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>PR, Advertising &amp; Marketing Jobs</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850982908?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=9DCE9674F9157B9847C1633926793B81F6701C2D</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>6b930f9eb1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Shubhda Bhutra Architecture + Design</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>junior, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5849890034?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=5B0039C8AFF10B97E207203A412D3A5659ED3B16</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>da7bcbe8c9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>21</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>HR Yaar</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>junior, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5825674656?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=714CA1A6B6BF672A9BD5B6DD56FFC51EDACC1EB2</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0b5f27f9ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>21</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Z Carbon Studios</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>junior, india (place)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5840225160?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=07E2649854F41DDE730A2B4888E890D4A9990B9D</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>03e7cc6952</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>21</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Junior Editor</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outwrk</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>junior, india (place)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850982953?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F8F7FD4235AEC7A32BAF89C9FB95BED02693D91B</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>cb531e647d</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>21</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Rohaan Constructions Private Limited</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>junior, chennai (place)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5833435233?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7FBF73F37474FD3A38A6EF54DDE95237EF78F1A1</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>bd98921cde</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Pure Cube Design Studio</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>junior, hyderabad (place)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5837737517?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=9BB41B08D8E6D7D3FFF6C5DDE9D8B079564A8F43</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>d9e2011ea7</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Junior Copywriter</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tonic Worldwide</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>junior, india (place)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5846297991?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7DAEAB2C4EFFADE8B0CFABF4D85EE2080AF408AA</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>5f5aad61a7</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>21</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Junior Architect</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Poetry Designs</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>junior, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5846663301?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C1A874118526E731BED59E1296E1A0820B6B13E3</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>4ec787347a</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>21</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Junior Copywriter</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Publicis Groupe</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>junior, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>PR, Advertising &amp; Marketing Jobs</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5743507573?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=8DFF4BE4EE12111EE2AB0B7FD81FAE481181B100</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>80cc4176cf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>21</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Junior Lighting Designer</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Keus Smart Home</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>junior, hyderabad (place)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5846663300?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2D5864CF70E7D2E7BFD63833A5FB920296CCD4D5</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>5112d02d10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>21</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Junior Video Editor</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>junior, mumbai (place)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5845682891?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=6E76E44BF412FCAA7240B046C4727984EB5C5846</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>6494ec9725</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>21</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Junior Video Editor</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Kickass Media Co.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>junior, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>PR, Advertising &amp; Marketing Jobs</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5848120301?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7BA79FCFB79A22D640BBDD1A46C6A372CE07E345</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ef7fef6851</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Junior Graphic Designer</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pixel Monkey</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>junior, chennai (place)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>PR, Advertising &amp; Marketing Jobs</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5845683248?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=59BF31F0BC2B57E6A3CFDEEB941E82C7EBCE2D2D</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>d8e606ad48</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>21</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Junior Sales Executive</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Trade W</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>junior, india (place)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Sales Jobs</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5841754901?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=9FF29814698958A6C5B975D92D9314951CE3633B</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>0ba200e4ec</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>21</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Junior Architect 2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ateliér ASRAYA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>junior, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Creative &amp; Design Jobs</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5848119687?se=zlwQznSd8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C048821677B5B16BE6FB476BD4F57FC78EB48650</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>f6827facaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>18</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Junior Scrum Master</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Vonage</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>junior, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Product, Full-Time</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/vonage-junior-scrum-master</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>9e2bd601cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>17</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GRC Analyst</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>analyst, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Front-End Programming, Full-Time</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/vercel-grc-analyst</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>51606110dd</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>16</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>16</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Zenara Health</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>engineer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>d592e60ddc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>16</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Precast Design Engineer</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fisher Associates, P.e., L.s., L.a., D.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>engineer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Design, Full-Time</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/fisher-associates-p-e-l-s-l-a-d-precast-design-engineer</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>35e1092dfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>16</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Customer Success Engineer</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Hightouch</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>engineer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Customer Support, Full-Time</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/hightouch-customer-success-engineer</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>7859de02e2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>16</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Tier III Service Desk Engineer</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Unio Digital</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Worldwide</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>remotive</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>engineer, worldwide (place)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Information Technology, full_time</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://remotive.com/remote-jobs/information-technology/tier-iii-service-desk-engineer-2091045</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>17f629b43a</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
         <v>7</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>engineer, remote (tag), remote (place)</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>

</xml_diff>

<commit_message>
Daily job scan: 2026-08-22
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -489,7 +489,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -532,37 +532,37 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138847?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=32DCB9AA4021747CA6EE87FF6C179711F6D6802D</t>
+          <t>https://www.adzuna.in/land/ad/5837138847?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=32DCB9AA4021747CA6EE87FF6C179711F6D6802D</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1f848feb07</t>
+          <t>3a5f96a677</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Software Engineer - Full Stack Development</t>
+          <t>.Net Python - AI Claude Developer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>full stack, software engineer, software, engineer, bangalore (place)</t>
+          <t>ai, python, developer, mumbai (place)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -582,42 +582,42 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138769?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2F7F009D1BCB621D977BBB3A9F3804F80C2B3BE1</t>
+          <t>https://www.adzuna.in/land/ad/5829141739?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F3FFF9BE552E9F66D6B6E4A05BB4B3A0CB091A87</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>c7ba77927b</t>
+          <t>b1b4418073</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>.Net Python - AI Claude Developer</t>
+          <t>Backend Developer- Python</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ai, python, developer, mumbai (place)</t>
+          <t>backend, python, developer, bangalore (place)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -637,37 +637,37 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5829141739?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F3FFF9BE552E9F66D6B6E4A05BB4B3A0CB091A87</t>
+          <t>https://www.adzuna.in/land/ad/5837138703?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=21D74D2D75ABF8D23E544DFE97E76A06BBA93975</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5323733872</t>
+          <t>f888fb79c2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Backend Developer- Python</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>backend, python, developer, bangalore (place)</t>
+          <t>ai, developer, bangalore (place)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -692,92 +692,92 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138703?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=21D74D2D75ABF8D23E544DFE97E76A06BBA93975</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>f4689f3991</t>
+          <t>4d63f38e87</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>full stack, engineer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>35</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>AI and Automation Developer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Bangalore, Karnataka</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>adzuna</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>ai, developer, bangalore (place)</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>IT Jobs</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5850906546?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0863155E89D7835B0B61ACA369B4495F6365687A</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1aec5c5501</t>
+          <t>cac067822e</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Full Stack Engineer</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Deutsche Bank</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>full stack, engineer, bangalore (place)</t>
+          <t>ai, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -802,42 +802,42 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850906546?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0863155E89D7835B0B61ACA369B4495F6365687A</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>af14cf91df</t>
+          <t>cf619e50e0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Full Stack Engineer, AVP</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Deutsche Bank</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>full stack, engineer, bangalore (place)</t>
+          <t>ai, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -857,97 +857,97 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723435?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E6F10ED3682D9E418B2752622F646D7D7C5C7099</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>eebe49a80e</t>
+          <t>56c5abfd7e</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>31</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>AI Solutions Engineer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Bangalore, Karnataka</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>adzuna</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ai, engineer, bangalore (place)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>IT Jobs</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>de99cb6309</t>
+          <t>f5887cf583</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Jr. Engineer Thermo Forming Machine Maintenace</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -957,27 +957,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ai, engineer, hyderabad (place)</t>
+          <t>engineer, india (place)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Engineering Jobs</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5785773010?se=cgNb8NWd8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=A00A57D5B4F42B3BE1314CCD60A59A74F015D9E7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9a9009a989</t>
+          <t>8731a712ab</t>
         </is>
       </c>
     </row>
@@ -988,51 +988,51 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Full Stack Software Engineer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ai, engineer, anywhere (place)</t>
+          <t>full stack, software engineer, software, engineer, india (place)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5837138847?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=32DCB9AA4021747CA6EE87FF6C179711F6D6802D</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>1f848feb07</t>
         </is>
       </c>
     </row>
@@ -1043,21 +1043,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Software Engineer - Full Stack Development</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>full stack, software engineer, software, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1077,17 +1077,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5837138769?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2F7F009D1BCB621D977BBB3A9F3804F80C2B3BE1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>c812a848de</t>
+          <t>c7ba77927b</t>
         </is>
       </c>
     </row>
@@ -1098,51 +1098,51 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>.Net Python - AI Claude Developer</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>ai, python, developer, mumbai (place)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5829141739?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F3FFF9BE552E9F66D6B6E4A05BB4B3A0CB091A87</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>5323733872</t>
         </is>
       </c>
     </row>
@@ -1153,49 +1153,544 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>48</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Backend Developer- Python</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Kyndryl</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>backend, python, developer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5837138703?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=21D74D2D75ABF8D23E544DFE97E76A06BBA93975</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>f4689f3991</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>35</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AI and Automation Developer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ai, developer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>1aec5c5501</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>32</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>full stack, engineer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850906546?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0863155E89D7835B0B61ACA369B4495F6365687A</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>af14cf91df</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>32</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer, AVP</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>full stack, engineer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5846723435?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E6F10ED3682D9E418B2752622F646D7D7C5C7099</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>eebe49a80e</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>31</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AI Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ai, engineer, bangalore (place)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>de99cb6309</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>31</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ai, engineer, hyderabad (place)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>9a9009a989</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>28</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Zenara Health</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ai, engineer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>d592e60ddc</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>23</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=KHzNDnad8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>c812a848de</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
         <v>6</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>engineer, remote (place)</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>

</xml_diff>

<commit_message>
Job scan: 2026-08-22 04:22 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1404,21 +1404,21 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1464,51 +1464,51 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -1524,49 +1524,109 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>22</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>11</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -1574,7 +1634,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-22 08:29 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -504,16 +504,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -528,27 +528,27 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -564,51 +564,51 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -624,36 +624,36 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -693,12 +693,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -718,17 +718,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -748,12 +748,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -808,17 +808,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -868,17 +868,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -928,17 +928,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -988,17 +988,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1008,27 +1008,27 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1068,27 +1068,27 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1143,12 +1143,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1164,21 +1164,21 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1224,21 +1224,21 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1464,21 +1464,21 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1498,17 +1498,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1524,51 +1524,51 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1584,49 +1584,229 @@
         </is>
       </c>
       <c r="C20" t="n">
+        <v>26</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Associate Instructor</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BeyondTrust</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>devops (tag), associate (level), anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>4c1963b96c</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>25</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>22</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>11</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -1634,7 +1814,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-22 12:37 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1284,21 +1284,21 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,27 +1308,27 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1498,17 +1498,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1584,51 +1584,51 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1644,51 +1644,51 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -1704,51 +1704,51 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -1764,49 +1764,109 @@
         </is>
       </c>
       <c r="C23" t="n">
+        <v>22</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>11</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -1814,7 +1874,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-22 18:30 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1344,51 +1344,51 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1618,17 +1618,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1644,51 +1644,51 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1704,51 +1704,51 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -1764,16 +1764,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1788,27 +1788,27 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -1824,49 +1824,169 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>25</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>22</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
         <v>11</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -1874,7 +1994,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-22 20:21 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1704,16 +1704,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1728,12 +1728,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -1764,36 +1764,36 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -1824,51 +1824,51 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -1884,51 +1884,51 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -1944,49 +1944,109 @@
         </is>
       </c>
       <c r="C26" t="n">
+        <v>22</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
         <v>11</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -1994,7 +2054,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-23 01:18 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -500,55 +500,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -564,16 +564,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -588,27 +588,27 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -624,51 +624,51 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -684,36 +684,36 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -808,12 +808,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -868,17 +868,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -928,17 +928,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -988,17 +988,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1048,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1068,27 +1068,27 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1108,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1128,27 +1128,27 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,27 +1308,27 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1344,36 +1344,36 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1404,51 +1404,51 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1618,17 +1618,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1678,17 +1678,17 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1704,51 +1704,51 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1764,16 +1764,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -1824,36 +1824,36 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -1884,51 +1884,51 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -1944,51 +1944,51 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2004,49 +2004,109 @@
         </is>
       </c>
       <c r="C27" t="n">
+        <v>22</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>11</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2054,7 +2114,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-23 06:40 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -560,55 +560,55 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -624,16 +624,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -648,27 +648,27 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -684,51 +684,51 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -744,36 +744,36 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -783,12 +783,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -813,12 +813,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -868,12 +868,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -928,17 +928,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -988,17 +988,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1048,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,17 +1078,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,27 +1128,27 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1168,12 +1168,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1188,27 +1188,27 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1263,12 +1263,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,27 +1368,27 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1404,36 +1404,36 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1464,51 +1464,51 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1623,12 +1623,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1678,17 +1678,17 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1738,17 +1738,17 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1764,51 +1764,51 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1824,16 +1824,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -1884,36 +1884,36 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -1944,51 +1944,51 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2004,51 +2004,51 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2064,49 +2064,109 @@
         </is>
       </c>
       <c r="C28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
         <v>11</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2114,7 +2174,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-23 08:29 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -564,51 +564,51 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -620,55 +620,55 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -684,16 +684,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -708,27 +708,27 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -744,51 +744,51 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -804,36 +804,36 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -988,17 +988,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1048,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,17 +1078,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,27 +1188,27 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1228,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1248,27 +1248,27 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,27 +1428,27 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1464,36 +1464,36 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1524,51 +1524,51 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1623,12 +1623,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1738,17 +1738,17 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1798,17 +1798,17 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1824,51 +1824,51 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1884,16 +1884,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -1944,36 +1944,36 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2004,51 +2004,51 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2064,51 +2064,51 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2124,49 +2124,109 @@
         </is>
       </c>
       <c r="C29" t="n">
+        <v>22</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>11</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2174,7 +2234,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-23 18:28 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -680,55 +680,55 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -744,16 +744,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -768,27 +768,27 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -804,51 +804,51 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -864,36 +864,36 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -933,12 +933,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -988,12 +988,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1048,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,17 +1078,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,27 +1248,27 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1288,12 +1288,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1308,27 +1308,27 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,27 +1488,27 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1524,36 +1524,36 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1584,51 +1584,51 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1798,17 +1798,17 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1858,17 +1858,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1884,51 +1884,51 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -1944,16 +1944,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1968,12 +1968,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2004,36 +2004,36 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2064,51 +2064,51 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2124,51 +2124,51 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2184,49 +2184,109 @@
         </is>
       </c>
       <c r="C30" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
         <v>11</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2234,7 +2294,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-24 01:16 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -500,55 +500,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Java Software Develper Engineer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CSG</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>61</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DESARROLLADOR FULL STACK</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>remoteok</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -564,51 +564,51 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -624,51 +624,51 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -684,16 +684,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -708,27 +708,27 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -740,55 +740,55 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -804,16 +804,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -828,27 +828,27 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -864,51 +864,51 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -924,36 +924,36 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -963,12 +963,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,17 +1078,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,27 +1308,27 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1348,12 +1348,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1368,27 +1368,27 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1498,17 +1498,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1548,27 +1548,27 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1584,36 +1584,36 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1623,12 +1623,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1644,51 +1644,51 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1858,17 +1858,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1918,17 +1918,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -1944,51 +1944,51 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2004,16 +2004,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2028,12 +2028,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2064,36 +2064,36 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2103,12 +2103,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2124,51 +2124,51 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2184,51 +2184,51 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2244,49 +2244,109 @@
         </is>
       </c>
       <c r="C31" t="n">
+        <v>22</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
         <v>11</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2294,7 +2354,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-24 08:48 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -560,55 +560,55 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -624,51 +624,51 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -684,51 +684,51 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -744,16 +744,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -768,27 +768,27 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -800,55 +800,55 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -864,16 +864,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -888,27 +888,27 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -924,51 +924,51 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -984,36 +984,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1053,12 +1053,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,17 +1078,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1108,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,27 +1368,27 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1428,27 +1428,27 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1608,27 +1608,27 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1644,36 +1644,36 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1704,51 +1704,51 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1918,17 +1918,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1978,17 +1978,17 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2004,51 +2004,51 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2064,16 +2064,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2088,12 +2088,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2103,12 +2103,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2124,36 +2124,36 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2163,12 +2163,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2184,51 +2184,51 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2244,51 +2244,51 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2304,49 +2304,109 @@
         </is>
       </c>
       <c r="C32" t="n">
+        <v>22</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
         <v>11</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2354,7 +2414,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-24 10:37 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -564,36 +564,36 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -603,12 +603,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -620,55 +620,55 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -684,51 +684,51 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -744,51 +744,51 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -804,16 +804,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -828,27 +828,27 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -860,55 +860,55 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -924,16 +924,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -948,27 +948,27 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -984,51 +984,51 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1044,36 +1044,36 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1138,17 +1138,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1168,12 +1168,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,27 +1428,27 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1468,12 +1468,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1488,27 +1488,27 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1618,17 +1618,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1648,17 +1648,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1668,27 +1668,27 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1704,36 +1704,36 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1764,51 +1764,51 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1978,17 +1978,17 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2038,17 +2038,17 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2064,51 +2064,51 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2124,16 +2124,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2163,12 +2163,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2184,36 +2184,36 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2244,51 +2244,51 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2304,51 +2304,51 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2364,49 +2364,109 @@
         </is>
       </c>
       <c r="C33" t="n">
+        <v>22</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
         <v>11</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2414,7 +2474,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-24 20:29 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -504,51 +504,51 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -564,21 +564,21 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -588,27 +588,27 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -624,36 +624,36 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -680,55 +680,55 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -744,51 +744,51 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -804,51 +804,51 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -864,16 +864,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -888,27 +888,27 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -920,55 +920,55 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -984,16 +984,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1008,27 +1008,27 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1044,51 +1044,51 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1104,36 +1104,36 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1143,12 +1143,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1173,12 +1173,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1228,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1258,17 +1258,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,27 +1488,27 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1548,27 +1548,27 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1623,12 +1623,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1648,17 +1648,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1678,17 +1678,17 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1708,17 +1708,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1728,27 +1728,27 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1764,36 +1764,36 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1824,51 +1824,51 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2038,17 +2038,17 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2098,17 +2098,17 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2124,51 +2124,51 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2184,16 +2184,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2208,12 +2208,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2244,36 +2244,36 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2283,12 +2283,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2304,51 +2304,51 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2364,51 +2364,51 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2424,49 +2424,109 @@
         </is>
       </c>
       <c r="C34" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
         <v>11</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2474,7 +2534,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 01:14 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -500,55 +500,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI/RAG engineer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CoinMarketCap</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Worldwide</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>79</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Standard Chartered Bank</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Bangalore, Karnataka</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>adzuna</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>data scientist, ai, bangalore (place)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>IT Jobs</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -560,55 +560,55 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -624,51 +624,51 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -684,51 +684,51 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -740,55 +740,55 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -800,20 +800,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -828,27 +828,27 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -864,36 +864,36 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -924,36 +924,36 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -963,12 +963,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -980,55 +980,55 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1040,55 +1040,55 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1104,51 +1104,51 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1164,21 +1164,21 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1224,51 +1224,51 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1498,17 +1498,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1548,27 +1548,27 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1618,17 +1618,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1648,17 +1648,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1668,27 +1668,27 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1708,17 +1708,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1738,17 +1738,17 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1768,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1788,27 +1788,27 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1824,51 +1824,51 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -1884,21 +1884,21 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1908,27 +1908,27 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -1944,51 +1944,51 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2098,17 +2098,17 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2163,12 +2163,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2184,51 +2184,51 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2244,51 +2244,51 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2304,36 +2304,36 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2343,12 +2343,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2364,51 +2364,51 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2424,16 +2424,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2448,27 +2448,27 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2484,49 +2484,169 @@
         </is>
       </c>
       <c r="C35" t="n">
+        <v>25</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
         <v>11</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2534,7 +2654,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 05:36 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -620,55 +620,55 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -680,55 +680,55 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -744,51 +744,51 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -804,51 +804,51 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -860,55 +860,55 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -920,20 +920,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -948,27 +948,27 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -984,36 +984,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1044,36 +1044,36 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1100,55 +1100,55 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1160,55 +1160,55 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1224,51 +1224,51 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1284,21 +1284,21 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1344,51 +1344,51 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1408,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1618,17 +1618,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1648,12 +1648,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1668,27 +1668,27 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1708,17 +1708,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1738,17 +1738,17 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1768,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1788,27 +1788,27 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1828,17 +1828,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1858,17 +1858,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1888,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1908,27 +1908,27 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -1944,51 +1944,51 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2004,21 +2004,21 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2028,27 +2028,27 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2064,51 +2064,51 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2163,12 +2163,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2218,17 +2218,17 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2283,12 +2283,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2304,51 +2304,51 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2364,51 +2364,51 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2424,36 +2424,36 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2463,12 +2463,12 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2484,51 +2484,51 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2544,16 +2544,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2568,27 +2568,27 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2604,49 +2604,169 @@
         </is>
       </c>
       <c r="C37" t="n">
+        <v>25</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>22</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
         <v>11</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2654,7 +2774,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 05:50 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,21 +413,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,45 +449,50 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>years_required</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>company</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>posted</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -506,47 +512,48 @@
       <c r="C2" t="n">
         <v>60</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>AI/RAG engineer</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>CoinMarketCap</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Worldwide</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>d199d5cdfc</t>
         </is>
@@ -566,47 +573,48 @@
       <c r="C3" t="n">
         <v>42</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Icarus Digital Marketing</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>ai, anywhere (place)</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>60c87a59fd</t>
         </is>
@@ -626,47 +634,48 @@
       <c r="C4" t="n">
         <v>25</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Percona</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>cloud, india (place)</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>a97ee1ce9b</t>
         </is>
@@ -686,47 +695,48 @@
       <c r="C5" t="n">
         <v>17</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Techno Vista Dynamics</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>APAC,Middle East</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>workingnomads</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>0bde4f9b82</t>
         </is>
@@ -746,47 +756,48 @@
       <c r="C6" t="n">
         <v>79</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Standard Chartered Bank</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Bangalore, Karnataka</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>3130787ee8</t>
         </is>
@@ -806,47 +817,48 @@
       <c r="C7" t="n">
         <v>57</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Java Software Develper Engineer</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>CSG</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>7626a2cdd6</t>
         </is>
@@ -866,47 +878,48 @@
       <c r="C8" t="n">
         <v>42</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Android Software Engineer</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Hudson Manpower</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Worldwide</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>afb7954487</t>
         </is>
@@ -926,47 +939,48 @@
       <c r="C9" t="n">
         <v>22</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Application Security Engineer II</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Abnormal</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>dc9a51cdbc</t>
         </is>
@@ -986,47 +1000,48 @@
       <c r="C10" t="n">
         <v>61</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Not listed</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>911da99485</t>
         </is>
@@ -1046,47 +1061,48 @@
       <c r="C11" t="n">
         <v>42</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
         <is>
           <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>ai, anywhere (place)</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Product, Full-Time</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>a0e38d6b98</t>
         </is>
@@ -1106,47 +1122,48 @@
       <c r="C12" t="n">
         <v>35</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Salesforce Developer</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>bbbc562c11</t>
         </is>
@@ -1166,47 +1183,48 @@
       <c r="C13" t="n">
         <v>22</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
         <is>
           <t>IT Systems Administrator</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Ralliant</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>a720a38bd1</t>
         </is>
@@ -1226,47 +1244,48 @@
       <c r="C14" t="n">
         <v>79</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>ABB</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Bangalore, Karnataka</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>5ee47ace79</t>
         </is>
@@ -1286,47 +1305,48 @@
       <c r="C15" t="n">
         <v>64</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
         <is>
           <t>AI and Automation Developer</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Bangalore, Karnataka</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>98337240aa</t>
         </is>
@@ -1346,47 +1366,48 @@
       <c r="C16" t="n">
         <v>58</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
         <is>
           <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Zenara Health</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>d592e60ddc</t>
         </is>
@@ -1406,47 +1427,48 @@
       <c r="C17" t="n">
         <v>49</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Data Scientist</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Morningstar</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Mumbai, Maharashtra</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>data scientist, mumbai (place)</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>c46d670134</t>
         </is>
@@ -1466,47 +1488,48 @@
       <c r="C18" t="n">
         <v>49</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Data Scientist</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Kyndryl</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>data scientist, india (place)</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>39dacd7158</t>
         </is>
@@ -1526,47 +1549,48 @@
       <c r="C19" t="n">
         <v>49</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Data Science Instructor</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>data science, india (place)</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>660701d5cb</t>
         </is>
@@ -1586,47 +1610,48 @@
       <c r="C20" t="n">
         <v>49</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Cornerstone OnDemand</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Hyderabad, Telangana</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>c2ca14412d</t>
         </is>
@@ -1646,47 +1671,48 @@
       <c r="C21" t="n">
         <v>49</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Data Scientist</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Jabil</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>data scientist, india (place)</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>1a0dea6270</t>
         </is>
@@ -1706,47 +1732,48 @@
       <c r="C22" t="n">
         <v>49</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
         <is>
           <t>AI Solutions Engineer</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Bangalore, Karnataka</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>a2c0a3fc16</t>
         </is>
@@ -1766,47 +1793,48 @@
       <c r="C23" t="n">
         <v>49</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Part time Data Science Instructor</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>upGrad</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>data science, india (place)</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Part time Jobs</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>fa169c0060</t>
         </is>
@@ -1826,47 +1854,48 @@
       <c r="C24" t="n">
         <v>49</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Novartis</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>engineer, ai, india (place)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>3fd60b2320</t>
         </is>
@@ -1886,47 +1915,48 @@
       <c r="C25" t="n">
         <v>49</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>MSCI</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Mumbai, Maharashtra</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>43f406da07</t>
         </is>
@@ -1946,47 +1976,48 @@
       <c r="C26" t="n">
         <v>49</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Data Scientist - People Analytics</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>ABB</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Bangalore, Karnataka</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>data scientist, bangalore (place)</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>187dc9c03e</t>
         </is>
@@ -2006,47 +2037,48 @@
       <c r="C27" t="n">
         <v>49</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
         <is>
           <t>Data Science Instructor</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Hyderabad, Telangana</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>data science, hyderabad (place)</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Teaching Jobs</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
           <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>5c41be551e</t>
         </is>
@@ -2066,47 +2098,48 @@
       <c r="C28" t="n">
         <v>48</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
         <is>
           <t>PHP Developer - Work From Home</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>CC Staffing International</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K28" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>14b619fb91</t>
         </is>
@@ -2126,47 +2159,48 @@
       <c r="C29" t="n">
         <v>45</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
         <is>
           <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>RWS</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>ai, delhi (place)</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>bb43fd7b08</t>
         </is>
@@ -2186,47 +2220,48 @@
       <c r="C30" t="n">
         <v>45</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
         <is>
           <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>RWS</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>ai, delhi (place)</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>fe688433d1</t>
         </is>
@@ -2246,47 +2281,48 @@
       <c r="C31" t="n">
         <v>45</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
         <is>
           <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>RWS</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>ai, delhi (place)</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>91c279dfff</t>
         </is>
@@ -2306,47 +2342,48 @@
       <c r="C32" t="n">
         <v>45</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
         <is>
           <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>RWS</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>ai, delhi (place)</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>170ea3eac1</t>
         </is>
@@ -2366,47 +2403,48 @@
       <c r="C33" t="n">
         <v>45</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
         <is>
           <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>RWS</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>ai, delhi (place)</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>616fb76ab0</t>
         </is>
@@ -2426,47 +2464,48 @@
       <c r="C34" t="n">
         <v>34</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>mercor</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K34" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
           <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>be05dc52ff</t>
         </is>
@@ -2486,47 +2525,48 @@
       <c r="C35" t="n">
         <v>30</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
         <is>
           <t>AWS Authorized Instructor</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>ITC WORLDWIDE</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>himalayas</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K35" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
           <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>a42ddc7b02</t>
         </is>
@@ -2546,47 +2586,48 @@
       <c r="C36" t="n">
         <v>26</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
         <is>
           <t>Associate Instructor</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>BeyondTrust</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
       <c r="K36" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
           <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>4c1963b96c</t>
         </is>
@@ -2606,47 +2647,48 @@
       <c r="C37" t="n">
         <v>25</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
         <is>
           <t>E-learning Developer</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Crowe UAE</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>adzuna</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>developer, ahmedabad (place)</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>IT Jobs</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>843701dc9e</t>
         </is>
@@ -2666,47 +2708,48 @@
       <c r="C38" t="n">
         <v>22</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
         <is>
           <t>Developer Educator</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>PlanetScale</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Anywhere in the World</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>weworkremotely</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>developer, anywhere (place)</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>c72ab4031d</t>
         </is>
@@ -2726,47 +2769,48 @@
       <c r="C39" t="n">
         <v>11</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 08:41 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -571,17 +571,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -632,37 +632,37 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -693,52 +693,52 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -750,56 +750,56 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -815,52 +815,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -876,22 +876,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -901,27 +901,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -937,37 +937,37 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -994,56 +994,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1059,52 +1059,52 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1120,52 +1120,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1181,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1206,27 +1206,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1238,56 +1238,56 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1303,17 +1303,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1328,27 +1328,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1364,52 +1364,52 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1425,37 +1425,37 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1552,12 +1552,12 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1582,17 +1582,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1613,17 +1613,17 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1643,17 +1643,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1674,17 +1674,17 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1704,17 +1704,17 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1765,17 +1765,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1796,17 +1796,17 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1816,27 +1816,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1953,12 +1953,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -1979,17 +1979,17 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2009,17 +2009,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2040,17 +2040,17 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2060,27 +2060,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2096,37 +2096,37 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2136,12 +2136,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2157,52 +2157,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2223,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2258,12 +2258,12 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2375,17 +2375,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2436,17 +2436,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2462,52 +2462,52 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2523,17 +2523,17 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2584,37 +2584,37 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2624,12 +2624,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2645,52 +2645,52 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2706,52 +2706,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -2767,50 +2767,111 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>11</v>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2818,7 +2879,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 14:44 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -571,52 +571,52 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -632,52 +632,52 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -693,37 +693,37 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -754,52 +754,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -811,56 +811,56 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -872,56 +872,56 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -937,52 +937,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -998,52 +998,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1055,56 +1055,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1116,21 +1116,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1145,27 +1145,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1181,37 +1181,37 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1221,12 +1221,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1242,37 +1242,37 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1299,56 +1299,56 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1360,56 +1360,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1425,52 +1425,52 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1486,22 +1486,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1547,52 +1547,52 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1613,17 +1613,17 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1643,17 +1643,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1674,17 +1674,17 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1735,12 +1735,12 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1765,17 +1765,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1796,17 +1796,17 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -1979,17 +1979,17 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1999,27 +1999,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2040,17 +2040,17 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2101,17 +2101,17 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2121,27 +2121,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2157,52 +2157,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2218,22 +2218,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2279,52 +2279,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2380,12 +2380,12 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2436,17 +2436,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2523,52 +2523,52 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2584,52 +2584,52 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2645,37 +2645,37 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2685,12 +2685,12 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2706,52 +2706,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2767,17 +2767,17 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2792,27 +2792,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2828,50 +2828,172 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>22</v>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>11</v>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -2879,7 +3001,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-25 16:37 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -693,52 +693,52 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -754,52 +754,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -815,37 +815,37 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -876,52 +876,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -933,56 +933,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -994,56 +994,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1059,52 +1059,52 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1120,52 +1120,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1177,56 +1177,56 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1238,21 +1238,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1267,27 +1267,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1303,37 +1303,37 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1343,12 +1343,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1364,37 +1364,37 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1421,56 +1421,56 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1482,56 +1482,56 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1547,52 +1547,52 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1608,22 +1608,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1643,17 +1643,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1669,52 +1669,52 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1765,17 +1765,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1796,17 +1796,17 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1887,17 +1887,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1999,27 +1999,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2040,17 +2040,17 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2101,17 +2101,17 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2121,27 +2121,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2162,17 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2192,17 +2192,17 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2223,17 +2223,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2279,52 +2279,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2340,22 +2340,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2365,27 +2365,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2401,52 +2401,52 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2558,17 +2558,17 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2624,12 +2624,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2645,52 +2645,52 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2706,52 +2706,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2767,37 +2767,37 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2807,12 +2807,12 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2828,52 +2828,52 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2889,17 +2889,17 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2914,27 +2914,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -2950,50 +2950,172 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>22</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>11</v>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3001,7 +3123,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-26 01:17 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,56 +506,56 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -571,52 +571,52 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -657,27 +657,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -698,17 +698,17 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -718,27 +718,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -794,12 +794,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -815,52 +815,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -937,37 +937,37 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -998,52 +998,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -1055,56 +1055,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1120,52 +1120,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1181,22 +1181,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1206,27 +1206,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1242,37 +1242,37 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1299,56 +1299,56 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1364,52 +1364,52 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1425,52 +1425,52 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1486,17 +1486,17 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1511,27 +1511,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1543,56 +1543,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1608,17 +1608,17 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1633,27 +1633,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1669,52 +1669,52 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1730,37 +1730,37 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1770,12 +1770,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -1801,12 +1801,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1887,17 +1887,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -1979,17 +1979,17 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2009,17 +2009,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -2040,17 +2040,17 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2101,17 +2101,17 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2121,27 +2121,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2162,12 +2162,12 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2182,27 +2182,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2223,17 +2223,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2258,12 +2258,12 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2284,17 +2284,17 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2314,17 +2314,17 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2365,27 +2365,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2401,37 +2401,37 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2441,12 +2441,12 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2462,52 +2462,52 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2624,12 +2624,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2680,17 +2680,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2741,17 +2741,17 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -2767,52 +2767,52 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -2828,17 +2828,17 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2853,12 +2853,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2868,12 +2868,12 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -2889,37 +2889,37 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2929,12 +2929,12 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -2950,52 +2950,52 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -3011,52 +3011,52 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -3072,50 +3072,111 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>11</v>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3123,7 +3184,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-26 04:39 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -567,21 +567,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -596,27 +596,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -628,56 +628,56 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -689,56 +689,56 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -750,56 +750,56 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -815,52 +815,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -876,52 +876,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -937,52 +937,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -998,52 +998,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -1059,52 +1059,52 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -1116,56 +1116,56 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -1177,56 +1177,56 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -1238,26 +1238,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1267,27 +1267,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -1299,56 +1299,56 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1360,56 +1360,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1421,41 +1421,41 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1482,26 +1482,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1511,27 +1511,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1552,47 +1552,47 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1604,56 +1604,56 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1665,56 +1665,56 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1726,56 +1726,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1787,56 +1787,56 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1852,22 +1852,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1913,22 +1913,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -1974,52 +1974,52 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -2045,12 +2045,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -2101,17 +2101,17 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2131,17 +2131,17 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -2162,12 +2162,12 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2187,22 +2187,22 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -2223,17 +2223,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2253,17 +2253,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -2284,17 +2284,17 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2375,17 +2375,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2406,17 +2406,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2426,27 +2426,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2462,17 +2462,17 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2523,22 +2523,22 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2584,22 +2584,22 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2619,17 +2619,17 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2645,22 +2645,22 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2670,27 +2670,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2706,52 +2706,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2807,12 +2807,12 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2828,52 +2828,52 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2889,52 +2889,52 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -2950,52 +2950,52 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -3011,22 +3011,22 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3046,17 +3046,17 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -3072,52 +3072,52 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -3133,50 +3133,294 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
+          <t>AWS Authorized Instructor</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ITC WORLDWIDE</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>cloud (tag), aws, india (place)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>a42ddc7b02</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>26</v>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Associate Instructor</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BeyondTrust</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>devops (tag), associate (level), anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>4c1963b96c</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>25</v>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>22</v>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>11</v>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3184,7 +3428,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-26 08:42 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -754,37 +754,39 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -794,12 +796,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -811,21 +813,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -840,27 +842,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -876,52 +878,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -942,12 +944,12 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -962,27 +964,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -1003,17 +1005,17 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1023,27 +1025,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -1069,12 +1071,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1084,7 +1086,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1099,12 +1101,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -1120,52 +1122,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1183,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1206,7 +1208,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1221,12 +1223,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -1242,37 +1244,37 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1282,12 +1284,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -1303,52 +1305,52 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -1360,56 +1362,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1425,52 +1427,52 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1486,22 +1488,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1511,27 +1513,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1547,37 +1549,37 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1587,12 +1589,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1604,56 +1606,56 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1669,52 +1671,52 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1730,52 +1732,52 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1791,17 +1793,17 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1816,27 +1818,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1848,56 +1850,56 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -1913,17 +1915,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1938,27 +1940,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -1974,52 +1976,52 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -2035,37 +2037,37 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2075,12 +2077,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2108,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2121,7 +2123,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2131,17 +2133,17 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -2162,12 +2164,12 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2182,7 +2184,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2192,17 +2194,17 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -2223,17 +2225,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2243,7 +2245,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2253,17 +2255,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -2284,17 +2286,17 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2304,7 +2306,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2314,17 +2316,17 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2347,17 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2365,7 +2367,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2375,17 +2377,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2406,17 +2408,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2426,27 +2428,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2467,12 +2469,12 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2487,27 +2489,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2528,17 +2530,17 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2548,7 +2550,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2563,12 +2565,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2589,17 +2591,17 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2609,7 +2611,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2619,17 +2621,17 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2650,17 +2652,17 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2670,27 +2672,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2706,37 +2708,37 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2746,12 +2748,12 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2767,52 +2769,52 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2835,7 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2868,12 +2870,12 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2896,7 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2929,12 +2931,12 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2957,7 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2985,17 +2987,17 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3018,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3046,17 +3048,17 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -3072,52 +3074,52 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -3133,17 +3135,17 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3158,12 +3160,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3173,12 +3175,12 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -3194,37 +3196,37 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3234,12 +3236,12 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -3255,52 +3257,52 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -3316,52 +3318,52 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -3377,50 +3379,111 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>11</v>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3428,7 +3491,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-26 12:51 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -754,19 +754,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -781,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -796,12 +794,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -817,37 +815,37 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -857,12 +855,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -874,56 +872,58 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -935,56 +935,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -1000,52 +1000,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -1066,17 +1066,17 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1096,17 +1096,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -1127,17 +1127,17 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1147,27 +1147,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -1183,52 +1183,52 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -1244,52 +1244,52 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -1305,37 +1305,37 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1345,12 +1345,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -1366,52 +1366,52 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -1423,56 +1423,56 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -1484,56 +1484,56 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1549,52 +1549,52 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1610,52 +1610,52 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1667,56 +1667,56 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1728,21 +1728,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1757,27 +1757,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1793,37 +1793,37 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1854,37 +1854,37 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -1911,56 +1911,56 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -1972,56 +1972,56 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -2037,52 +2037,52 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -2098,22 +2098,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -2159,52 +2159,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -2225,17 +2225,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2255,17 +2255,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -2286,17 +2286,17 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -2347,12 +2347,12 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2377,17 +2377,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -2408,17 +2408,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2438,17 +2438,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2469,12 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2489,27 +2489,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2530,17 +2530,17 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2560,17 +2560,17 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2591,17 +2591,17 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2611,27 +2611,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2652,17 +2652,17 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2682,17 +2682,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2713,17 +2713,17 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2733,27 +2733,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2769,52 +2769,52 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2830,22 +2830,22 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2855,27 +2855,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -2891,52 +2891,52 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2992,12 +2992,12 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3048,17 +3048,17 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -3135,52 +3135,52 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -3196,52 +3196,52 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -3257,37 +3257,37 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3297,12 +3297,12 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -3318,52 +3318,52 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -3379,17 +3379,17 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3404,27 +3404,27 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -3440,50 +3440,172 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>22</v>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>11</v>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3491,7 +3613,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-26 16:48 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -571,37 +571,37 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -759,32 +759,32 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -794,12 +794,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -876,19 +876,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -903,12 +901,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -918,12 +916,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -939,17 +937,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -964,12 +962,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -979,12 +977,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -996,56 +994,58 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>60</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -1057,56 +1057,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -1122,52 +1122,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -1188,17 +1188,17 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1218,17 +1218,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -1249,17 +1249,17 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1269,27 +1269,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -1305,52 +1305,52 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -1366,52 +1366,52 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -1427,37 +1427,37 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -1488,52 +1488,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -1545,56 +1545,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -1606,56 +1606,56 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -1671,52 +1671,52 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -1732,52 +1732,52 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -1789,56 +1789,56 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -1850,21 +1850,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1879,27 +1879,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -1915,37 +1915,37 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -1976,37 +1976,37 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2016,12 +2016,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -2033,56 +2033,56 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -2094,56 +2094,56 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -2159,52 +2159,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -2220,22 +2220,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2255,17 +2255,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -2281,52 +2281,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -2347,17 +2347,17 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2377,17 +2377,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -2408,17 +2408,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2443,12 +2443,12 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2469,12 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2499,17 +2499,17 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -2530,17 +2530,17 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2560,17 +2560,17 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2611,27 +2611,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -2652,17 +2652,17 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2682,17 +2682,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -2713,17 +2713,17 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2733,27 +2733,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -2774,17 +2774,17 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2804,17 +2804,17 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -2835,17 +2835,17 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2855,27 +2855,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -2891,52 +2891,52 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -2952,22 +2952,22 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2977,27 +2977,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -3013,52 +3013,52 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3170,17 +3170,17 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3236,12 +3236,12 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -3257,52 +3257,52 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -3318,52 +3318,52 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -3379,37 +3379,37 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3419,12 +3419,12 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -3440,52 +3440,52 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -3501,17 +3501,17 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3526,27 +3526,27 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -3562,50 +3562,172 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>22</v>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>11</v>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3613,7 +3735,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-27 07:48 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,26 +506,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -545,17 +545,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -576,17 +576,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -628,56 +628,56 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -689,56 +689,56 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -750,56 +750,56 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -811,21 +811,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -840,27 +840,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -872,21 +872,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -901,27 +901,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -937,52 +937,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -998,39 +998,37 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1040,12 +1038,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1059,12 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1086,7 +1084,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1101,12 +1099,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1118,21 +1116,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1147,27 +1145,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1179,56 +1177,56 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -1240,56 +1238,56 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -1301,56 +1299,56 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -1362,56 +1360,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -1423,21 +1421,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>46</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1452,27 +1452,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -1484,56 +1484,56 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -1549,22 +1549,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1574,27 +1574,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -1610,52 +1610,52 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -1667,26 +1667,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1696,27 +1696,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -1728,56 +1728,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -1789,56 +1789,56 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -1850,21 +1850,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1879,27 +1879,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -1911,56 +1911,56 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -1972,56 +1972,56 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2033,56 +2033,56 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2094,56 +2094,56 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2155,56 +2155,56 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -2216,56 +2216,56 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -2277,21 +2277,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2316,17 +2316,17 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -2338,56 +2338,56 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -2399,56 +2399,56 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -2460,21 +2460,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2484,32 +2484,32 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -2521,56 +2521,56 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -2586,22 +2586,22 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2626,12 +2626,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -2647,12 +2647,12 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2682,17 +2682,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -2708,52 +2708,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -2774,17 +2774,17 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2804,17 +2804,17 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -2835,17 +2835,17 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2865,17 +2865,17 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2926,17 +2926,17 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2977,27 +2977,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3013,17 +3013,17 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3033,32 +3033,32 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3074,22 +3074,22 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3109,17 +3109,17 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3135,22 +3135,22 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3160,27 +3160,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3196,22 +3196,22 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3236,12 +3236,12 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -3257,22 +3257,22 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3292,17 +3292,17 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -3318,22 +3318,22 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -3379,37 +3379,37 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3419,12 +3419,12 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -3440,17 +3440,17 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3480,12 +3480,12 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -3501,52 +3501,52 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -3562,22 +3562,22 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3597,17 +3597,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -3623,52 +3623,52 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -3684,50 +3684,477 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
+          <t>AI Data Specialist - Hindi</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>RWS</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>ai, delhi (place)</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>170ea3eac1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>45</v>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>AI Data Specialist - Tamil</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>RWS</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ai, delhi (place)</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>616fb76ab0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>34</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>mercor</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>engineer, ai (tag), india (place)</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>be05dc52ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>30</v>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>AWS Authorized Instructor</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ITC WORLDWIDE</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>cloud (tag), aws, india (place)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>a42ddc7b02</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>26</v>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Associate Instructor</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BeyondTrust</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>devops (tag), associate (level), anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>4c1963b96c</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>25</v>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>22</v>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>11</v>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H61" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="J61" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="M61" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -3735,7 +4162,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-27 18:53 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -571,22 +571,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -642,12 +642,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -733,12 +733,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -794,12 +794,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -815,37 +815,37 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -876,52 +876,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -933,56 +933,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -994,56 +994,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1055,41 +1055,41 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1116,41 +1116,41 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1160,12 +1160,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1181,52 +1181,52 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1242,37 +1242,37 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1308,32 +1308,32 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1343,12 +1343,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1369,12 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1425,39 +1425,37 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1467,12 +1465,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -1488,37 +1486,37 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1528,12 +1526,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -1545,56 +1543,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -1606,56 +1604,56 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -1667,56 +1665,58 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>49</v>
-      </c>
-      <c r="D21" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -1728,56 +1728,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -1793,52 +1793,52 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -1854,52 +1854,52 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -1915,52 +1915,52 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -1976,52 +1976,52 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -2037,52 +2037,52 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -2094,56 +2094,56 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -2155,56 +2155,56 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -2216,26 +2216,26 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2245,27 +2245,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2277,56 +2277,56 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2338,56 +2338,56 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2399,41 +2399,41 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2443,12 +2443,12 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -2460,26 +2460,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2489,27 +2489,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2530,47 +2530,47 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -2582,56 +2582,56 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -2643,56 +2643,56 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -2704,56 +2704,56 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -2765,56 +2765,56 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -2830,22 +2830,22 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2855,27 +2855,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -2891,22 +2891,22 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2926,17 +2926,17 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -2952,52 +2952,52 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -3023,12 +3023,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3048,17 +3048,17 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -3079,17 +3079,17 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3109,17 +3109,17 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -3140,12 +3140,12 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3165,22 +3165,22 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3231,17 +3231,17 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3262,17 +3262,17 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3297,12 +3297,12 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3323,12 +3323,12 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3384,17 +3384,17 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3404,27 +3404,27 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3440,17 +3440,17 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3460,32 +3460,32 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -3501,22 +3501,22 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -3562,22 +3562,22 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3597,17 +3597,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -3623,22 +3623,22 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3648,27 +3648,27 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -3684,52 +3684,52 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3785,12 +3785,12 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -3806,52 +3806,52 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -3867,52 +3867,52 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -3928,52 +3928,52 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -3989,22 +3989,22 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4024,17 +4024,17 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -4050,52 +4050,52 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -4111,50 +4111,294 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
+          <t>AWS Authorized Instructor</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ITC WORLDWIDE</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>cloud (tag), aws, india (place)</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>a42ddc7b02</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>26</v>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Associate Instructor</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>BeyondTrust</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>devops (tag), associate (level), anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>4c1963b96c</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>25</v>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>22</v>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>11</v>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -4162,7 +4406,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-28 18:15 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,56 +506,56 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Data Scientist - AI &amp; Automation</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>data scientist, automation, ai, bangalore (place)</t>
+          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2e19a4f3f6</t>
+          <t>17936ac69e</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -576,17 +576,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MTS-1 Machine Learning Engineer</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>machine learning, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
+          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>c65fcd065c</t>
+          <t>a8bcca74c0</t>
         </is>
       </c>
     </row>
@@ -628,26 +628,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Machine Learning Engineer (T25)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>e99054d24c</t>
         </is>
       </c>
     </row>
@@ -689,16 +689,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>SWE-3 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>83e0ebd10e</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -759,17 +759,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -794,12 +794,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>ec1b34ae37</t>
         </is>
       </c>
     </row>
@@ -811,56 +811,56 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>AI Data Annotator - Remote</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Argos Multilingual Inc.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>All Other Remote, Contract</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>5c22526a85</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Data Scientist with R programming</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -911,17 +911,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>dbec4a04a4</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -937,37 +937,37 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -998,52 +998,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -1059,52 +1059,52 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Education Designer UX UI and AI</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>design, content writing, education</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ca62234445</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -1120,52 +1120,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Course Writer and Editor UX UI and AI</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>design, content writing</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>01210e4343</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -1177,26 +1177,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1216,17 +1216,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1247,17 +1247,17 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1277,17 +1277,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -1299,56 +1299,56 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -1360,56 +1360,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1421,41 +1421,41 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1482,41 +1482,41 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1547,52 +1547,52 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1608,37 +1608,37 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1648,12 +1648,12 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1669,39 +1669,37 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>40</v>
-      </c>
-      <c r="D21" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1711,12 +1709,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1730,12 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1757,7 +1755,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1772,12 +1770,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1789,21 +1787,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1818,27 +1816,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -1850,56 +1848,56 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -1911,56 +1909,56 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -1972,56 +1970,56 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -2033,56 +2031,58 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>49</v>
-      </c>
-      <c r="D27" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -2094,56 +2094,56 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -2159,52 +2159,52 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -2220,52 +2220,52 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -2281,52 +2281,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -2338,26 +2338,26 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2377,17 +2377,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -2399,56 +2399,56 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -2460,56 +2460,56 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -2521,21 +2521,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2550,27 +2550,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -2582,56 +2582,56 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2643,56 +2643,56 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2704,56 +2704,56 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2765,21 +2765,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -2826,56 +2826,56 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -2887,56 +2887,56 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -2948,56 +2948,56 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -3009,56 +3009,56 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -3070,21 +3070,21 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3094,32 +3094,32 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -3131,21 +3131,21 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3155,32 +3155,32 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -3196,22 +3196,22 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3221,27 +3221,27 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -3257,22 +3257,22 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3292,17 +3292,17 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -3318,37 +3318,37 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -3384,17 +3384,17 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3404,27 +3404,27 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -3445,12 +3445,12 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3475,17 +3475,17 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -3506,17 +3506,17 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3536,17 +3536,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -3567,17 +3567,17 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3597,17 +3597,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3628,17 +3628,17 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3648,27 +3648,27 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3684,52 +3684,52 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3745,22 +3745,22 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3770,27 +3770,27 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3806,22 +3806,22 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3846,12 +3846,12 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -3867,22 +3867,22 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3907,12 +3907,12 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -3928,22 +3928,22 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3963,17 +3963,17 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -3989,22 +3989,22 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4014,27 +4014,27 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -4050,17 +4050,17 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4075,12 +4075,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4090,12 +4090,12 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -4111,52 +4111,52 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -4172,52 +4172,52 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -4233,22 +4233,22 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -4268,17 +4268,17 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -4294,52 +4294,52 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -4355,50 +4355,416 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
+          <t>AI Data Specialist - Tamil</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>RWS</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>ai, delhi (place)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>616fb76ab0</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>34</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>mercor</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>engineer, ai (tag), india (place)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>be05dc52ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>30</v>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>AWS Authorized Instructor</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ITC WORLDWIDE</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>himalayas</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>cloud (tag), aws, india (place)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>a42ddc7b02</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>26</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Associate Instructor</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>BeyondTrust</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>devops (tag), associate (level), anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>DevOps and Sysadmin, Full-Time</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>4c1963b96c</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>25</v>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>E-learning Developer</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Crowe UAE</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>adzuna</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>developer, ahmedabad (place)</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>IT Jobs</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>843701dc9e</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>22</v>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>11</v>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L71" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="M71" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -4406,7 +4772,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-29 10:51 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,56 +506,58 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>38</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Backend Software Engineer, PDP Experience</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
+          <t>software engineer, backend, anywhere (place)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
+          <t>Back-End Programming, Full-Time</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
+          <t>https://weworkremotely.com/remote-jobs/reddit-backend-software-engineer-pdp-experience</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>17936ac69e</t>
+          <t>a954ce85ab</t>
         </is>
       </c>
     </row>
@@ -571,37 +573,37 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>machine learning, engineer, hyderabad (place)</t>
+          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -611,12 +613,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>a8bcca74c0</t>
+          <t>17936ac69e</t>
         </is>
       </c>
     </row>
@@ -637,17 +639,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer (T25)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -657,7 +659,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>machine learning, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -667,17 +669,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
+          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>e99054d24c</t>
+          <t>a8bcca74c0</t>
         </is>
       </c>
     </row>
@@ -698,7 +700,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SWE-3 Machine Learning Engineer</t>
+          <t>Machine Learning Engineer (T25)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -733,12 +735,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
+          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>83e0ebd10e</t>
+          <t>e99054d24c</t>
         </is>
       </c>
     </row>
@@ -754,22 +756,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>SWE-3 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -779,7 +781,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -794,12 +796,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
+          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ec1b34ae37</t>
+          <t>83e0ebd10e</t>
         </is>
       </c>
     </row>
@@ -815,52 +817,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AI Data Annotator - Remote</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Argos Multilingual Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>All Other Remote, Contract</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
+          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>5c22526a85</t>
+          <t>ec1b34ae37</t>
         </is>
       </c>
     </row>
@@ -872,56 +874,56 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Data Scientist - AI &amp; Automation</t>
+          <t>AI Data Annotator - Remote</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Argos Multilingual Inc.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>data scientist, automation, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>All Other Remote, Contract</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
+          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2e19a4f3f6</t>
+          <t>5c22526a85</t>
         </is>
       </c>
     </row>
@@ -937,12 +939,12 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MTS-1 Machine Learning Engineer</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -962,7 +964,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -977,12 +979,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>c65fcd065c</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -998,22 +1000,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1023,7 +1025,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1033,17 +1035,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -1069,12 +1071,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1084,7 +1086,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1094,17 +1096,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -1160,12 +1162,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1188,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1221,12 +1223,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1249,12 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Scientist with R programming</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1277,17 +1279,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>dbec4a04a4</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -1303,52 +1305,52 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1406,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -1425,52 +1427,52 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Education Designer UX UI and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>design, content writing, education</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ca62234445</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1493,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Course Writer and Editor UX UI and AI</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1516,7 +1518,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>design, content writing</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1526,12 +1528,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>01210e4343</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1543,56 +1545,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1608,17 +1610,17 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1633,7 +1635,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1643,17 +1645,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1669,37 +1671,37 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1709,12 +1711,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1737,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1770,12 +1772,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1798,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1831,12 +1833,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1857,32 +1859,32 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1892,12 +1894,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1920,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1953,12 +1955,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -1979,32 +1981,32 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2014,12 +2016,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -2035,39 +2037,37 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>40</v>
-      </c>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -2098,37 +2098,39 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20</v>
-      </c>
-      <c r="D28" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2138,12 +2140,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -2155,21 +2157,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2184,27 +2186,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -2220,52 +2222,52 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2288,12 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2306,27 +2308,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -2347,17 +2349,17 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2367,27 +2369,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2415,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2428,7 +2430,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2443,12 +2445,12 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -2464,52 +2466,52 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -2525,17 +2527,17 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2550,7 +2552,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2565,12 +2567,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -2586,37 +2588,37 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2626,12 +2628,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -2647,52 +2649,52 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2704,56 +2706,56 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2769,52 +2771,52 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2830,22 +2832,22 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2855,27 +2857,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -2891,37 +2893,37 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2931,12 +2933,12 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -2948,56 +2950,56 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -3013,52 +3015,52 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -3074,52 +3076,52 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -3135,17 +3137,17 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3160,27 +3162,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -3192,56 +3194,56 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3259,17 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3282,27 +3284,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -3318,52 +3320,52 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -3379,37 +3381,37 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3419,12 +3421,12 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -3450,12 +3452,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3465,7 +3467,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3475,17 +3477,17 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3508,12 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3526,7 +3528,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3536,17 +3538,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -3567,17 +3569,17 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3587,7 +3589,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3597,17 +3599,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -3628,17 +3630,17 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3648,7 +3650,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3658,17 +3660,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3689,17 +3691,17 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3709,7 +3711,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3719,17 +3721,17 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3750,17 +3752,17 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3770,27 +3772,27 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3811,12 +3813,12 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3831,27 +3833,27 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3872,17 +3874,17 @@
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3892,7 +3894,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3907,12 +3909,12 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -3933,17 +3935,17 @@
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3953,7 +3955,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3963,17 +3965,17 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -3994,17 +3996,17 @@
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4014,27 +4016,27 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -4050,37 +4052,37 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4090,12 +4092,12 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -4111,52 +4113,52 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4179,7 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4212,12 +4214,12 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4240,7 @@
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4273,12 +4275,12 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4301,7 @@
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4329,17 +4331,17 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4362,7 @@
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4390,17 +4392,17 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -4416,52 +4418,52 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -4477,17 +4479,17 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4502,12 +4504,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4517,12 +4519,12 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -4538,37 +4540,37 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4578,12 +4580,12 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -4599,52 +4601,52 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -4660,52 +4662,52 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -4721,50 +4723,111 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>11</v>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="I72" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="J72" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
+      <c r="K72" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr">
+      <c r="L72" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="M72" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -4772,7 +4835,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-29 16:17 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -569,16 +569,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Open Source Contributor</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -598,27 +598,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
+          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
+          <t>Open-Source-Contributor, Open-Source-Developer, Open-Source-Software-Developer, Open-Source-Advocate, Open-Source-Engineer, Open-Source-Software-Engineer, Open-Source-Software-Maintainer, Community-Contributor, Entry-level</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
+          <t>https://himalayas.app/companies/micro1/jobs/open-source-contributor-4150550716</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>17936ac69e</t>
+          <t>d8033bd793</t>
         </is>
       </c>
     </row>
@@ -634,37 +634,37 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>machine learning, engineer, hyderabad (place)</t>
+          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>a8bcca74c0</t>
+          <t>17936ac69e</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer (T25)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>machine learning, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -730,17 +730,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
+          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>e99054d24c</t>
+          <t>a8bcca74c0</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SWE-3 Machine Learning Engineer</t>
+          <t>Machine Learning Engineer (T25)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
+          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>83e0ebd10e</t>
+          <t>e99054d24c</t>
         </is>
       </c>
     </row>
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>SWE-3 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -857,12 +857,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
+          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ec1b34ae37</t>
+          <t>83e0ebd10e</t>
         </is>
       </c>
     </row>
@@ -878,52 +878,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI Data Annotator - Remote</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Argos Multilingual Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>All Other Remote, Contract</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
+          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>5c22526a85</t>
+          <t>ec1b34ae37</t>
         </is>
       </c>
     </row>
@@ -935,56 +935,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Data Scientist - AI &amp; Automation</t>
+          <t>AI Data Annotator - Remote</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Argos Multilingual Inc.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>data scientist, automation, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>All Other Remote, Contract</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
+          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2e19a4f3f6</t>
+          <t>5c22526a85</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MTS-1 Machine Learning Engineer</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1040,12 +1040,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>c65fcd065c</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -1061,22 +1061,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1096,17 +1096,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1157,17 +1157,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -1223,12 +1223,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1310,12 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Data Scientist with R programming</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1340,17 +1340,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>dbec4a04a4</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -1366,52 +1366,52 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -1467,12 +1467,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -1488,52 +1488,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Education Designer UX UI and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>design, content writing, education</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ca62234445</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Course Writer and Editor UX UI and AI</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>design, content writing</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>01210e4343</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1606,56 +1606,56 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1671,17 +1671,17 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1706,17 +1706,17 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1732,37 +1732,37 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1920,32 +1920,32 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2016,12 +2016,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -2042,32 +2042,32 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -2098,39 +2098,37 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>40</v>
-      </c>
-      <c r="D28" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2140,12 +2138,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -2161,37 +2159,39 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>20</v>
-      </c>
-      <c r="D29" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -2218,21 +2218,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2247,27 +2247,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -2283,52 +2283,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -2349,12 +2349,12 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2369,27 +2369,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -2410,17 +2410,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2430,27 +2430,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -2476,12 +2476,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2506,12 +2506,12 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -2527,52 +2527,52 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -2588,17 +2588,17 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -2649,37 +2649,37 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -2710,52 +2710,52 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2767,56 +2767,56 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2832,52 +2832,52 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2893,22 +2893,22 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2918,27 +2918,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -2954,37 +2954,37 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -3011,56 +3011,56 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -3076,52 +3076,52 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -3137,52 +3137,52 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -3198,17 +3198,17 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3223,27 +3223,27 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -3255,56 +3255,56 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -3320,17 +3320,17 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3345,27 +3345,27 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -3381,52 +3381,52 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -3442,37 +3442,37 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3482,12 +3482,12 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -3513,12 +3513,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3538,17 +3538,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3599,17 +3599,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -3630,17 +3630,17 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3660,17 +3660,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -3691,17 +3691,17 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3752,17 +3752,17 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3782,17 +3782,17 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3813,17 +3813,17 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3833,27 +3833,27 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3874,12 +3874,12 @@
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3894,27 +3894,27 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3935,17 +3935,17 @@
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3970,12 +3970,12 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -3996,17 +3996,17 @@
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4026,17 +4026,17 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -4057,17 +4057,17 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4077,27 +4077,27 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -4113,37 +4113,37 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -4174,52 +4174,52 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4275,12 +4275,12 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4336,12 +4336,12 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4392,17 +4392,17 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4453,17 +4453,17 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -4479,52 +4479,52 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -4540,17 +4540,17 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4565,12 +4565,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4580,12 +4580,12 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -4601,37 +4601,37 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4641,12 +4641,12 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -4662,52 +4662,52 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -4723,52 +4723,52 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -4784,50 +4784,111 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>11</v>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="M73" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -4835,7 +4896,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-30 09:51 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -506,58 +506,56 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>38</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Backend Software Engineer, PDP Experience</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>software engineer, backend, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Back-End Programming, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/reddit-backend-software-engineer-pdp-experience</t>
+          <t>https://www.adzuna.in/land/ad/5857982687?se=BGNyWVik8RGF59teMJsS7Q&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=64C652991D92D5E3DCA4519D688756F962092321</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>a954ce85ab</t>
+          <t>dd6de0380a</t>
         </is>
       </c>
     </row>
@@ -573,37 +571,39 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>38</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Open Source Contributor</t>
+          <t>Backend Software Engineer, PDP Experience</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
+          <t>software engineer, backend, anywhere (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Open-Source-Contributor, Open-Source-Developer, Open-Source-Software-Developer, Open-Source-Advocate, Open-Source-Engineer, Open-Source-Software-Engineer, Open-Source-Software-Maintainer, Community-Contributor, Entry-level</t>
+          <t>Back-End Programming, Full-Time</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/open-source-contributor-4150550716</t>
+          <t>https://weworkremotely.com/remote-jobs/reddit-backend-software-engineer-pdp-experience</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>d8033bd793</t>
+          <t>a954ce85ab</t>
         </is>
       </c>
     </row>
@@ -630,16 +630,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Open Source Contributor</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -659,27 +659,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
+          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
+          <t>Open-Source-Contributor, Open-Source-Developer, Open-Source-Software-Developer, Open-Source-Advocate, Open-Source-Engineer, Open-Source-Software-Engineer, Open-Source-Software-Maintainer, Community-Contributor, Entry-level</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
+          <t>https://himalayas.app/companies/micro1/jobs/open-source-contributor-4150550716</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>17936ac69e</t>
+          <t>d8033bd793</t>
         </is>
       </c>
     </row>
@@ -695,37 +695,37 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>machine learning, engineer, hyderabad (place)</t>
+          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,12 +735,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>a8bcca74c0</t>
+          <t>17936ac69e</t>
         </is>
       </c>
     </row>
@@ -761,17 +761,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer (T25)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>machine learning, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -791,17 +791,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
+          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>e99054d24c</t>
+          <t>a8bcca74c0</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SWE-3 Machine Learning Engineer</t>
+          <t>Machine Learning Engineer (T25)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -857,12 +857,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
+          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>83e0ebd10e</t>
+          <t>e99054d24c</t>
         </is>
       </c>
     </row>
@@ -878,22 +878,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>SWE-3 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
+          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ec1b34ae37</t>
+          <t>83e0ebd10e</t>
         </is>
       </c>
     </row>
@@ -939,52 +939,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Data Annotator - Remote</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Argos Multilingual Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>All Other Remote, Contract</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
+          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>5c22526a85</t>
+          <t>ec1b34ae37</t>
         </is>
       </c>
     </row>
@@ -996,56 +996,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Scientist - AI &amp; Automation</t>
+          <t>AI Data Annotator - Remote</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Argos Multilingual Inc.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data scientist, automation, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>All Other Remote, Contract</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
+          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2e19a4f3f6</t>
+          <t>5c22526a85</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MTS-1 Machine Learning Engineer</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>c65fcd065c</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1157,17 +1157,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1193,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1218,17 +1218,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -1284,12 +1284,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1345,12 +1345,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -1371,12 +1371,12 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Data Scientist with R programming</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1401,17 +1401,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>dbec4a04a4</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -1427,52 +1427,52 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -1549,52 +1549,52 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Education Designer UX UI and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>design, content writing, education</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ca62234445</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Course Writer and Editor UX UI and AI</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>design, content writing</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>01210e4343</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1667,56 +1667,56 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1732,17 +1732,17 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1767,17 +1767,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1793,37 +1793,37 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>162d6a9ed2</t>
+          <t>bb930fc93f</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
+          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/financial-accuracy-tax-logic-expert-ai-community-7007868696</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>637c85a300</t>
+          <t>162d6a9ed2</t>
         </is>
       </c>
     </row>
@@ -1981,32 +1981,32 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Education Designer: UX, UI, and AI</t>
+          <t>Identity Trust &amp; Fraud Intelligence Specialist - Intermediate (AI Community)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>IxDF - Interaction Design Foundation</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Design, Full-Time</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2016,12 +2016,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/identity-trust-fraud-intelligence-specialist-intermediate-ai-community</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>9fbe655de3</t>
+          <t>637c85a300</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Course Writer and Editor: UX, UI, and AI</t>
+          <t>Education Designer: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-education-designer-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>e8e07f5951</t>
+          <t>9fbe655de3</t>
         </is>
       </c>
     </row>
@@ -2103,32 +2103,32 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AI Consulting Domain Expert</t>
+          <t>Course Writer and Editor: UX, UI, and AI</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>IxDF - Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
+          <t>Design, Full-Time</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
+          <t>https://weworkremotely.com/remote-jobs/ixdf-interaction-design-foundation-course-writer-and-editor-ux-ui-and-ai</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>7f1041d829</t>
+          <t>e8e07f5951</t>
         </is>
       </c>
     </row>
@@ -2159,39 +2159,37 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>40</v>
-      </c>
-      <c r="D29" t="n">
-        <v>2</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
+          <t>AI Consulting Domain Expert</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>full stack, software, engineer, anywhere (place)</t>
+          <t>ai, worldwide (place)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Full-Stack Programming, Full-Time</t>
+          <t>AI-Domain-Expert, AI-Consultant, AI-Subject-Matter-Expert, Artificial-Intelligence-Consulting, Senior</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2201,12 +2199,12 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-consulting-domain-expert-7128968890</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>6fe968b6b9</t>
+          <t>7f1041d829</t>
         </is>
       </c>
     </row>
@@ -2222,37 +2220,39 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20</v>
-      </c>
-      <c r="D30" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>QA Speech-to-Text Audio Collection Project</t>
+          <t>Software Development Engineer II Full Stack - Business (Remote @ Colombia)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>qa, worldwide (place)</t>
+          <t>full stack, software, engineer, anywhere (place)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>Full-Stack Programming, Full-Time</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
+          <t>https://weworkremotely.com/remote-jobs/offerup-software-development-engineer-ii-full-stack-business-remote-colombia</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>a44e738ec6</t>
+          <t>6fe968b6b9</t>
         </is>
       </c>
     </row>
@@ -2279,21 +2279,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AI/RAG engineer</t>
+          <t>QA Speech-to-Text Audio Collection Project</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CoinMarketCap</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2308,27 +2308,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>engineer, ai, ml (tag), worldwide (place)</t>
+          <t>qa, worldwide (place)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
+          <t>Entry-level</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
+          <t>https://himalayas.app/companies/telus-digital/jobs/qa-speech-to-text-audio-collection-project</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>d199d5cdfc</t>
+          <t>a44e738ec6</t>
         </is>
       </c>
     </row>
@@ -2344,52 +2344,52 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>AI/RAG engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>CoinMarketCap</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>RAG-AI-Engineer, Machine-Learning-Engineering, AI-Engineering, RAG-Development, Vector-Search-Engineer, IA-RAG-Engineer, AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
+          <t>https://himalayas.app/companies/coinmarketcap/jobs/ai-rag-engineer</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>faa646b456</t>
+          <t>d199d5cdfc</t>
         </is>
       </c>
     </row>
@@ -2410,12 +2410,12 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data Science-Index Quant Specialist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2430,27 +2430,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>data science, mumbai (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
+          <t>https://www.adzuna.in/land/ad/5846723676?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F83D2913763A01EA6FBE321571CA8B989BE3F382</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>6ec3848d0b</t>
+          <t>faa646b456</t>
         </is>
       </c>
     </row>
@@ -2471,17 +2471,17 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Science-Index Quant Specialist</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2491,27 +2491,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>data scientist, gurgaon (place)</t>
+          <t>data science, mumbai (place)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Accounting &amp; Finance Jobs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
+          <t>https://www.adzuna.in/land/ad/5843137505?se=zow8fZOg8RGratEa7ObxPA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=EC4079028ED7338B991CD57034DE9EA5AC8D9A0B</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>e2cd9eda9e</t>
+          <t>6ec3848d0b</t>
         </is>
       </c>
     </row>
@@ -2537,12 +2537,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Gurgaon, Haryana</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>data scientist, delhi (place)</t>
+          <t>data scientist, gurgaon (place)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2567,12 +2567,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
+          <t>https://www.adzuna.in/land/ad/5849297019?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=E87B9A5E2A9605281144BBEA53533DB7165D1FA0</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>83a3456095</t>
+          <t>e2cd9eda9e</t>
         </is>
       </c>
     </row>
@@ -2588,52 +2588,52 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>GTM AI Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Customer.io</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, delhi (place)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5848650875?se=9hBOPKOg8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4DF45BC4D3A230C0689E561399F3F0BA2C0FC825</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>19a2ae7abb</t>
+          <t>83a3456095</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Performance Creative Strategist and AI Producer</t>
+          <t>GTM AI Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Icarus Digital Marketing</t>
+          <t>Customer.io</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
+          <t>https://weworkremotely.com/remote-jobs/customer-io-gtm-ai-engineer</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>60c87a59fd</t>
+          <t>19a2ae7abb</t>
         </is>
       </c>
     </row>
@@ -2710,37 +2710,37 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
+          <t>Performance Creative Strategist and AI Producer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Percona</t>
+          <t>Icarus Digital Marketing</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>cloud, india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
+          <t>Sales and Marketing, Full-Time</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
+          <t>https://weworkremotely.com/remote-jobs/icarus-digital-marketing-performance-creative-strategist-and-ai-producer</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>a97ee1ce9b</t>
+          <t>60c87a59fd</t>
         </is>
       </c>
     </row>
@@ -2771,52 +2771,52 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Offensive Cybersecurity Engineer - Red Team</t>
+          <t>GTM Coordinator, Cloud Native (Talent Pool)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Techno Vista Dynamics</t>
+          <t>Percona</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>APAC,Middle East</t>
+          <t>Bulgaria, Croatia, Czechia, Greece, Hungary, India, Poland, Portugal, Spain</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>workingnomads</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>engineer, testing (tag), apac (place)</t>
+          <t>cloud, india (place)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Development, engineer,security,penetration testing</t>
+          <t>GTM-Coordinator, Talent-Community-Coordinator, Talent-Operations-Coordinator, Entry-level</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.workingnomads.com/job/go/1781770/</t>
+          <t>https://himalayas.app/companies/percona/jobs/gtm-coordinator-cloud-native-talent-pool</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>0bde4f9b82</t>
+          <t>a97ee1ce9b</t>
         </is>
       </c>
     </row>
@@ -2828,56 +2828,56 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
+          <t>Offensive Cybersecurity Engineer - Red Team</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank</t>
+          <t>Techno Vista Dynamics</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>APAC,Middle East</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>workingnomads</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>engineer, testing (tag), apac (place)</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Development, engineer,security,penetration testing</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
+          <t>https://www.workingnomads.com/job/go/1781770/</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>3130787ee8</t>
+          <t>0bde4f9b82</t>
         </is>
       </c>
     </row>
@@ -2893,52 +2893,52 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Java Software Develper Engineer</t>
+          <t>Human-Centered AI Data Scientist, Strategy and Talent</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>CSG</t>
+          <t>Standard Chartered Bank</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
+          <t>https://www.adzuna.in/land/ad/5837139276?se=1M6Kj_qf8RGoxpN31Vp7kA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C0F814CBDD0355075DDB000131DE4C8D130504ED</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>7626a2cdd6</t>
+          <t>3130787ee8</t>
         </is>
       </c>
     </row>
@@ -2954,22 +2954,22 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Android Software Engineer</t>
+          <t>Java Software Develper Engineer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Hudson Manpower</t>
+          <t>CSG</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2979,27 +2979,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
+          <t>programmer (tag), developer (tag), software, engineer, backend (tag), java, india (place)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
+          <t>Java-Development, Software-Engineer, Entry-Level-Software-Development, Backend-Development, Technical-Support, Java-Software-Engineer, Java-Developer, Java-Developer-Jobs, Java-Application-Developer, Java-Programmer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
+          <t>https://himalayas.app/companies/csg/jobs/java-software-develper-engineer</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>afb7954487</t>
+          <t>7626a2cdd6</t>
         </is>
       </c>
     </row>
@@ -3015,37 +3015,37 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Application Security Engineer II</t>
+          <t>Android Software Engineer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Hudson Manpower</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>engineer, devops (tag), anywhere (place)</t>
+          <t>software engineer, android, kotlin (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>Android-Software-Engineer, Mobile-Development, Android-Development, Software-Engineer, Kotlin, Android-Engineer, Android-Software-Engineering, Mobile-Android-Engineer, Android-Systems-Engineer, Android-Engineering, Mobile-Software-Engineer, Senior</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
+          <t>https://himalayas.app/companies/hudson-manpower/jobs/android-software-engineer</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>dc9a51cdbc</t>
+          <t>afb7954487</t>
         </is>
       </c>
     </row>
@@ -3072,56 +3072,56 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>DESARROLLADOR FULL STACK</t>
+          <t>Application Security Engineer II</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Kruger NearShore LLC - Rekluti</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
+          <t>engineer, devops (tag), anywhere (place)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
+          <t>https://weworkremotely.com/remote-jobs/abnormal-application-security-engineer-ii</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>911da99485</t>
+          <t>dc9a51cdbc</t>
         </is>
       </c>
     </row>
@@ -3137,52 +3137,52 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>AI Transformation Owner, Product &amp; Design</t>
+          <t>DESARROLLADOR FULL STACK</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GitLab</t>
+          <t>Kruger NearShore LLC - Rekluti</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>full stack, front end (tag), backend (tag), angular (tag), testing (tag), python (tag), golang (tag), devops (tag), cloud (tag), git (tag)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>full stack, front end, python, dev, testing, web dev, quality assurance, devops, c, cloud, nosql, git, flutter, angular, mobile, golang, backend, digital nomad</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
+          <t>https://remoteOK.com/remote-jobs/remote-desarrollador-full-stack-kruger-nearshore-llc-rekluti-1137062</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>a0e38d6b98</t>
+          <t>911da99485</t>
         </is>
       </c>
     </row>
@@ -3198,52 +3198,52 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Salesforce Developer</t>
+          <t>AI Transformation Owner, Product &amp; Design</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Forrester Research, Inc. (US)</t>
+          <t>GitLab</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>developer, software (tag), cloud (tag), india (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
+          <t>https://weworkremotely.com/remote-jobs/gitlab-ai-transformation-owner-product-design</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>bbbc562c11</t>
+          <t>a0e38d6b98</t>
         </is>
       </c>
     </row>
@@ -3259,17 +3259,17 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>IT Systems Administrator</t>
+          <t>Salesforce Developer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Ralliant</t>
+          <t>Forrester Research, Inc. (US)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3284,27 +3284,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>developer (tag), engineer (tag), india (place)</t>
+          <t>developer, software (tag), cloud (tag), india (place)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
+          <t>Salesforce-Developer, CRM-Developer, Salesforce-Administrator, Integration-Developer, Software-Developer, Salesforce-CRM-Developer, Salesforce-Application-Developer, Salesforce-Sales-Cloud-Developer, Salesforce-Development, Salesforce-Solutions-Developer, Salesforce-Platform-Developer, Salesforce-Apex-Developer, Force.Com-Developer, Mid-level</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
+          <t>https://himalayas.app/companies/forrester-research-inc-us/jobs/salesforce-developer-8148624472</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>a720a38bd1</t>
+          <t>bbbc562c11</t>
         </is>
       </c>
     </row>
@@ -3316,56 +3316,56 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
+          <t>IT Systems Administrator</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Ralliant</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>data scientist, ai, bangalore (place)</t>
+          <t>developer (tag), engineer (tag), india (place)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Energy, Oil &amp; Gas Jobs</t>
+          <t>Power-Platform-Engineer, Business-intelligence-Engineer, Analytics-Engineer, Microsoft-Fabric-Engineer, Power-BI-Developer, IT-Systems-Administrator, IT-System-Administrator, Systems-Administrator, IT-Systems-Administration, IT-Administrator, Systems-Support-Administrator, Mid-level</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
+          <t>https://himalayas.app/companies/ralliant/jobs/it-systems-administrator</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>5ee47ace79</t>
+          <t>a720a38bd1</t>
         </is>
       </c>
     </row>
@@ -3381,17 +3381,17 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>AI and Automation Developer</t>
+          <t>Talent Pool -FP&amp;A- Data Scientist / Analytics Specialist / Data &amp; AI Specialist</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3406,27 +3406,27 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>automation, developer, ai, bangalore (place)</t>
+          <t>data scientist, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Energy, Oil &amp; Gas Jobs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
+          <t>https://www.adzuna.in/land/ad/5785773115?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=888721B9EAAF876B1F079BC209DECF1099E63440</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>98337240aa</t>
+          <t>5ee47ace79</t>
         </is>
       </c>
     </row>
@@ -3442,52 +3442,52 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
+          <t>AI and Automation Developer</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Zenara Health</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>engineer, devops, ai, anywhere (place)</t>
+          <t>automation, developer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
+          <t>https://www.adzuna.in/land/ad/5847959817?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=44960F01CCAE33F814C0EF4448956DF38E8344F5</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>d592e60ddc</t>
+          <t>98337240aa</t>
         </is>
       </c>
     </row>
@@ -3503,37 +3503,37 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>DevOps &amp; Security Engineer - AI-Native Healthcare SaaS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Zenara Health</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>engineer, devops, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
+          <t>https://weworkremotely.com/remote-jobs/zenara-health-devops-security-engineer-ai-native-healthcare-saas</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>c46d670134</t>
+          <t>d592e60ddc</t>
         </is>
       </c>
     </row>
@@ -3574,12 +3574,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Morningstar</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3599,17 +3599,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
+          <t>https://www.adzuna.in/land/ad/5846723381?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F9660467E3895814968DA45F3A82EF6912496F70</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>39dacd7158</t>
+          <t>c46d670134</t>
         </is>
       </c>
     </row>
@@ -3630,12 +3630,12 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3660,17 +3660,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
+          <t>https://www.adzuna.in/land/ad/5837138848?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=86962F79F06A105F30676367582529277DE10978</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>660701d5cb</t>
+          <t>39dacd7158</t>
         </is>
       </c>
     </row>
@@ -3691,17 +3691,17 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
+          <t>https://www.adzuna.in/land/ad/5833434843?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=95E30E442ED8EDC695067D6ACDD8806A1A4DBE0E</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>c2ca14412d</t>
+          <t>660701d5cb</t>
         </is>
       </c>
     </row>
@@ -3752,17 +3752,17 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Jabil</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>data scientist, india (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3782,17 +3782,17 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
+          <t>https://www.adzuna.in/land/ad/5837139103?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=23D035D0F5CFDFF88D2FBA2CB9721442B70F9874</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>1a0dea6270</t>
+          <t>c2ca14412d</t>
         </is>
       </c>
     </row>
@@ -3813,17 +3813,17 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>AI Solutions Engineer</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Jabil</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>engineer, ai, bangalore (place)</t>
+          <t>data scientist, india (place)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3843,17 +3843,17 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
+          <t>https://www.adzuna.in/land/ad/5785773097?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=1AD120B3FB3DFBC7F01669BC535E68EC0F2123A3</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>a2c0a3fc16</t>
+          <t>1a0dea6270</t>
         </is>
       </c>
     </row>
@@ -3874,17 +3874,17 @@
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Part time Data Science Instructor</t>
+          <t>AI Solutions Engineer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3894,27 +3894,27 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>data science, india (place)</t>
+          <t>engineer, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Part time Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
+          <t>https://www.adzuna.in/land/ad/5846723241?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0084818D71681FAC4F572D55AE1C6BC637792931</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>fa169c0060</t>
+          <t>a2c0a3fc16</t>
         </is>
       </c>
     </row>
@@ -3935,12 +3935,12 @@
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
+          <t>Part time Data Science Instructor</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3955,27 +3955,27 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>engineer, ai, india (place)</t>
+          <t>data science, india (place)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>Part time Jobs</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
+          <t>https://www.adzuna.in/land/ad/5850983469?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0F708DAB080760E3C6FB3FC40EA3A64A7B0306D9</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>3fd60b2320</t>
+          <t>fa169c0060</t>
         </is>
       </c>
     </row>
@@ -3996,17 +3996,17 @@
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Agentic AI Engineer for AI &amp;DS, BSI</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>engineer, ai, mumbai (place)</t>
+          <t>engineer, ai, india (place)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4031,12 +4031,12 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
+          <t>https://www.adzuna.in/land/ad/5785771743?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F6DC64E0C8FB2D27FC25CBE24085394F367A2687</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>43f406da07</t>
+          <t>3fd60b2320</t>
         </is>
       </c>
     </row>
@@ -4057,17 +4057,17 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Data Scientist - People Analytics</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>engineer, ai, mumbai (place)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -4087,17 +4087,17 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
+          <t>https://www.adzuna.in/land/ad/5785773171?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2185A7049B5506DF1182A45172761BBEF73613FA</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>187dc9c03e</t>
+          <t>43f406da07</t>
         </is>
       </c>
     </row>
@@ -4118,17 +4118,17 @@
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>Data Scientist - People Analytics</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Itvedant Education Pvt. Ltd.</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4138,27 +4138,27 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Teaching Jobs</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
+          <t>https://www.adzuna.in/land/ad/5821999876?se=uNVelwOe8RGfQpohglHoaw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=08993CE6BE520CA2C34926E81E8CBB0072304E1F</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>5c41be551e</t>
+          <t>187dc9c03e</t>
         </is>
       </c>
     </row>
@@ -4174,37 +4174,37 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>PHP Developer - Work From Home</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>CC Staffing International</t>
+          <t>Itvedant Education Pvt. Ltd.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
+          <t>Teaching Jobs</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4214,12 +4214,12 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
+          <t>https://www.adzuna.in/land/ad/5852476426?se=NskdSSae8RGSb8VpDRDiVA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=2B7C55A3F795EE4D2F2D732844EDA9B4CAC3F128</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>14b619fb91</t>
+          <t>5c41be551e</t>
         </is>
       </c>
     </row>
@@ -4235,52 +4235,52 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Kannada</t>
+          <t>PHP Developer - Work From Home</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>RWS</t>
+          <t>CC Staffing International</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>ai, delhi (place)</t>
+          <t>developer, software (tag), engineer (tag), backend (tag), php, india (place)</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>PHP-Developer, Backend-Engineer, Web-Development, Software-Developer, Full-Stack-Developer, Remote-PHP-Developer, PHP-Software-Engineer, Backend-PHP-Developer, Remote-Web-Developer, Developer, Mid-level</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
+          <t>https://himalayas.app/companies/cc-staffing-international/jobs/php-developer-work-from-home</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>bb43fd7b08</t>
+          <t>14b619fb91</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Marathi</t>
+          <t>AI Data Specialist - Kannada</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4336,12 +4336,12 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
+          <t>https://www.adzuna.in/land/ad/5785772642?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=96F9E6C80B83A39F4F2C05268274FD2EBE13B037</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>fe688433d1</t>
+          <t>bb43fd7b08</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Telugu</t>
+          <t>AI Data Specialist - Marathi</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4397,12 +4397,12 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
+          <t>https://www.adzuna.in/land/ad/5785772098?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=B26B7FB6A299BC3A2BFD29BF94BF59C981A24A29</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>91c279dfff</t>
+          <t>fe688433d1</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Hindi</t>
+          <t>AI Data Specialist - Telugu</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4453,17 +4453,17 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
+          <t>https://www.adzuna.in/land/ad/5785770664?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=D13E17364CDB48C8A2B963F62AC42C33A76C021B</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>170ea3eac1</t>
+          <t>91c279dfff</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4484,7 @@
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>AI Data Specialist - Tamil</t>
+          <t>AI Data Specialist - Hindi</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -4514,17 +4514,17 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
+          <t>https://www.adzuna.in/land/ad/5795883387?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=38289BC2F5CA723017CE2916CC4536DEA978B9A6</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>616fb76ab0</t>
+          <t>170ea3eac1</t>
         </is>
       </c>
     </row>
@@ -4540,52 +4540,52 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
+          <t>AI Data Specialist - Tamil</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>mercor</t>
+          <t>RWS</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>engineer, ai (tag), india (place)</t>
+          <t>ai, delhi (place)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
+          <t>https://www.adzuna.in/land/ad/5785772320?se=xp3UHeGd8RGIEJB03vDchg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AB56F1DD143407CEE31E12C4126DC533B06A2AD3</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>be05dc52ff</t>
+          <t>616fb76ab0</t>
         </is>
       </c>
     </row>
@@ -4601,17 +4601,17 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>AWS Authorized Instructor</t>
+          <t>Agent Operations Engineer - Fully Remote | Upto $500/task Task based</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>ITC WORLDWIDE</t>
+          <t>mercor</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4626,12 +4626,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>cloud (tag), aws, india (place)</t>
+          <t>engineer, ai (tag), india (place)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
+          <t>Agent-Engineering, LLMOperations, AI-Engineering, AI-Operations, Machine-Learning-Engineering, AgentOps-Engineer, Agent-Orchestration-Engineer, AI-Agents-Engineer, Operations-Engineer, Remote-AI-Engineer, Mid-level</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4641,12 +4641,12 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
+          <t>https://himalayas.app/companies/mercor/jobs/agent-operations-engineer-fully-remote-upto-500-task-task-based</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>a42ddc7b02</t>
+          <t>be05dc52ff</t>
         </is>
       </c>
     </row>
@@ -4662,37 +4662,37 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Associate Instructor</t>
+          <t>AWS Authorized Instructor</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>BeyondTrust</t>
+          <t>ITC WORLDWIDE</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>India</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>devops (tag), associate (level), anywhere (place)</t>
+          <t>cloud (tag), aws, india (place)</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>DevOps and Sysadmin, Full-Time</t>
+          <t>AWS-Training, Cloud-Computing-Instructor, Technical-Trainer, AWS-Authorized-Instructor, Cloud-Education, AWS-Certification-Training, Cloud-Instructor, Cloud-Computing-Trainer, Senior</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4702,12 +4702,12 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
+          <t>https://himalayas.app/companies/itc-worldwide/jobs/aws-authorized-instructor</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>4c1963b96c</t>
+          <t>a42ddc7b02</t>
         </is>
       </c>
     </row>
@@ -4723,52 +4723,52 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>E-learning Developer</t>
+          <t>Associate Instructor</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Crowe UAE</t>
+          <t>BeyondTrust</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>developer, ahmedabad (place)</t>
+          <t>devops (tag), associate (level), anywhere (place)</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>DevOps and Sysadmin, Full-Time</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
+          <t>https://weworkremotely.com/remote-jobs/beyondtrust-associate-instructor</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>843701dc9e</t>
+          <t>4c1963b96c</t>
         </is>
       </c>
     </row>
@@ -4784,52 +4784,52 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Developer Educator</t>
+          <t>E-learning Developer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>PlanetScale</t>
+          <t>Crowe UAE</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>developer, anywhere (place)</t>
+          <t>developer, ahmedabad (place)</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Sales and Marketing, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+          <t>https://www.adzuna.in/land/ad/5850983902?se=aqlCTd-d8RGU6LIjyaRnwA&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=F927DE790D9874EE6BA8C142D15CF3A7A97BFA7E</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>c72ab4031d</t>
+          <t>843701dc9e</t>
         </is>
       </c>
     </row>
@@ -4845,50 +4845,111 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
+          <t>Developer Educator</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>PlanetScale</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Anywhere in the World</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>weworkremotely</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>developer, anywhere (place)</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Sales and Marketing, Full-Time</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com/remote-jobs/planetscale-developer-educator</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>c72ab4031d</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>11</v>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
           <t>Consultant Implementation Engineer</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>Harbor</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>remoteok</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>engineer, golang (tag), remote (place)</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>consulting, technical, accounting, legal, golang, engineer</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t>https://remoteOK.com/remote-jobs/remote-consultant-implementation-engineer-harbor-1136987</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="M74" t="inlineStr">
         <is>
           <t>f724e65bc8</t>
         </is>
@@ -4896,7 +4957,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
+    <dataValidation sqref="A2:A74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick one of: new, applied, skipped" prompt="Mark this job applied once you have applied." type="list">
       <formula1>"new,applied,skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Job scan: 2026-08-30 14:42 UTC
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -567,58 +567,56 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>38</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Backend Software Engineer, PDP Experience</t>
+          <t>GitHub Contributor</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>software engineer, backend, anywhere (place)</t>
+          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Back-End Programming, Full-Time</t>
+          <t>Open-Source-Contributor, Open-Source-Developer, Community-Contributor, Open-Source-Software-Developer, Open-Source-Engineer, Developer, Entry-level</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/reddit-backend-software-engineer-pdp-experience</t>
+          <t>https://himalayas.app/companies/micro1/jobs/github-contributor-2145210908</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>a954ce85ab</t>
+          <t>9bd86980fc</t>
         </is>
       </c>
     </row>
@@ -634,37 +632,39 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>38</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Open Source Contributor</t>
+          <t>Backend Software Engineer, PDP Experience</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
+          <t>software engineer, backend, anywhere (place)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Open-Source-Contributor, Open-Source-Developer, Open-Source-Software-Developer, Open-Source-Advocate, Open-Source-Engineer, Open-Source-Software-Engineer, Open-Source-Software-Maintainer, Community-Contributor, Entry-level</t>
+          <t>Back-End Programming, Full-Time</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/open-source-contributor-4150550716</t>
+          <t>https://weworkremotely.com/remote-jobs/reddit-backend-software-engineer-pdp-experience</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>d8033bd793</t>
+          <t>a954ce85ab</t>
         </is>
       </c>
     </row>
@@ -691,16 +691,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Open Source Contributor</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -720,27 +720,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
+          <t>developer (tag), software (tag), engineer (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
+          <t>Open-Source-Contributor, Open-Source-Developer, Open-Source-Software-Developer, Open-Source-Advocate, Open-Source-Engineer, Open-Source-Software-Engineer, Open-Source-Software-Maintainer, Community-Contributor, Entry-level</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
+          <t>https://himalayas.app/companies/micro1/jobs/open-source-contributor-4150550716</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>17936ac69e</t>
+          <t>d8033bd793</t>
         </is>
       </c>
     </row>
@@ -756,37 +756,37 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Worldwide</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>himalayas</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>machine learning, engineer, hyderabad (place)</t>
+          <t>engineer, python (tag), ai, ml (tag), worldwide (place)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>AI-Engineer, Artificial-Intelligence-Engineer, AI-ML-Engineer, AI-Engineering-Specialist, AI-Engineering, Artificial-Intelligence-Engineering, Python-AI-Engineer, AI-Engineering-Jobs, Mid-level</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
+          <t>https://himalayas.app/companies/micro1/jobs/ai-engineer-7982880650</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>a8bcca74c0</t>
+          <t>17936ac69e</t>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer (T25)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>machine learning, engineer, hyderabad (place)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -852,17 +852,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
+          <t>https://www.adzuna.in/land/ad/5859662671?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=77410E24CED3D457054E58156829472F42D5B958</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>e99054d24c</t>
+          <t>a8bcca74c0</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SWE-3 Machine Learning Engineer</t>
+          <t>Machine Learning Engineer (T25)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
+          <t>https://www.adzuna.in/land/ad/5858538850?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=AA8B404BB5F08B6BBBC1A1DAEA80EDAE2331BB01</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>83e0ebd10e</t>
+          <t>e99054d24c</t>
         </is>
       </c>
     </row>
@@ -939,22 +939,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>SWE-3 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>engineer, ai, hyderabad (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
+          <t>https://www.adzuna.in/land/ad/5858537539?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=49BEDAECA8CA01D8F7BFB9CA5D092D8DD046FCF4</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ec1b34ae37</t>
+          <t>83e0ebd10e</t>
         </is>
       </c>
     </row>
@@ -1000,52 +1000,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AI Data Annotator - Remote</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Argos Multilingual Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ai, anywhere (place)</t>
+          <t>engineer, ai, hyderabad (place)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>All Other Remote, Contract</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
+          <t>https://www.adzuna.in/land/ad/5857982475?se=nBIHegyj8RGmT-3sKckM2g&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=61932F7A965BC6190F96EF3EDD6B34FCA7CA0EFF</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>5c22526a85</t>
+          <t>ec1b34ae37</t>
         </is>
       </c>
     </row>
@@ -1057,56 +1057,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Data Scientist - AI &amp; Automation</t>
+          <t>AI Data Annotator - Remote</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Argos Multilingual Inc.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data scientist, automation, ai, bangalore (place)</t>
+          <t>ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>All Other Remote, Contract</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
+          <t>https://weworkremotely.com/remote-jobs/argos-multilingual-inc-ai-data-annotator-remote</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2e19a4f3f6</t>
+          <t>5c22526a85</t>
         </is>
       </c>
     </row>
@@ -1122,12 +1122,12 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MTS-1 Machine Learning Engineer</t>
+          <t>Data Scientist - AI &amp; Automation</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>machine learning, engineer, bangalore (place)</t>
+          <t>data scientist, automation, ai, bangalore (place)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
+          <t>https://www.adzuna.in/land/ad/5857251125?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=C7BA7BE347A1ADA1FC538497AF302C4F3AD6BEDD</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>c65fcd065c</t>
+          <t>2e19a4f3f6</t>
         </is>
       </c>
     </row>
@@ -1183,22 +1183,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>MTS-1 Machine Learning Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>data scientist, mumbai (place)</t>
+          <t>machine learning, engineer, bangalore (place)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1218,17 +1218,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
+          <t>https://www.adzuna.in/land/ad/5858537523?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=4219F9238C4FE19DFCEAD65DAA98E56A5B89F388</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>200651f002</t>
+          <t>c65fcd065c</t>
         </is>
       </c>
     </row>
@@ -1254,12 +1254,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data scientist, bangalore (place)</t>
+          <t>data scientist, mumbai (place)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1279,17 +1279,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
+          <t>https://www.adzuna.in/land/ad/5849296977?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=0FFA2BB725355D26B4B624FA5365F48C2D8B894C</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>6a6f7a8419</t>
+          <t>200651f002</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
+          <t>https://www.adzuna.in/land/ad/5857251146?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=43EC4FC89638B5AB4C3D5267B80E2B1135A6C706</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>aa6eef76e8</t>
+          <t>6a6f7a8419</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Data Scientist, Knowledge Management</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
+          <t>https://www.adzuna.in/land/ad/5857251173?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=7E2FD9B14C3A74461E2352F6CFE714131C13E4BC</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>d1497475d4</t>
+          <t>aa6eef76e8</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Data Scientist with R programming</t>
+          <t>Data Scientist, Knowledge Management</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1462,17 +1462,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
+          <t>https://www.adzuna.in/land/ad/5857251185?se=Epj_tuuh8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=74B3EB71D85FA01AB90B707F8DB6AB9F2A17FAFA</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>dbec4a04a4</t>
+          <t>d1497475d4</t>
         </is>
       </c>
     </row>
@@ -1488,52 +1488,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
+          <t>Data Scientist with R programming</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Anywhere in the World</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>weworkremotely</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>engineer, ai, anywhere (place)</t>
+          <t>data scientist, bangalore (place)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Product, Full-Time</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
+          <t>https://www.adzuna.in/land/ad/5837139433?se=OqwplEii8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=221D7BCDBBE6E4012ED68B71EDB34DB2E07507EC</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>e7de7648c1</t>
+          <t>dbec4a04a4</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer-1</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>dada5ade61</t>
+          <t>e7de7648c1</t>
         </is>
       </c>
     </row>
@@ -1610,52 +1610,52 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Education Designer UX UI and AI</t>
+          <t>AI Engineer - FDE (Forward Deployed Engineer)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Interaction Design Foundation</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>Anywhere in the World</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>remoteok</t>
+          <t>weworkremotely</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>engineer, ai, anywhere (place)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>design, content writing, education</t>
+          <t>Product, Full-Time</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
+          <t>https://weworkremotely.com/remote-jobs/databricks-ai-engineer-fde-forward-deployed-engineer</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ca62234445</t>
+          <t>dada5ade61</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Course Writer and Editor UX UI and AI</t>
+          <t>Education Designer UX UI and AI</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>design, content writing</t>
+          <t>design, content writing, education</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
+          <t>https://remoteOK.com/remote-jobs/remote-education-designer-ux-ui-and-ai-interaction-design-foundation-1137138</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>01210e4343</t>
+          <t>ca62234445</t>
         </is>
       </c>
     </row>
@@ -1728,56 +1728,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>App Developer - AI/ML</t>
+          <t>Course Writer and Editor UX UI and AI</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>Interaction Design Foundation</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>adzuna</t>
+          <t>remoteok</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>developer, ai, ml, hyderabad (place)</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>IT Jobs</t>
+          <t>design, content writing</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
+          <t>https://remoteOK.com/remote-jobs/remote-course-writer-and-editor-ux-ui-and-ai-interaction-design-foundation-1137136</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>7a22fe6bd5</t>
+          <t>01210e4343</t>
         </is>
       </c>
     </row>
@@ -1793,17 +1793,17 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Data Science Instructor</t>
+          <t>App Developer - AI/ML</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>upGrad</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>data science, hyderabad (place)</t>
+          <t>developer, ai, ml, hyderabad (place)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1828,17 +1828,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
+          <t>https://www.adzuna.in/land/ad/5837139469?se=-BSx1eug8RG-Sdz4qyZPjg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=16DC1893C3026AA51441662E0B1A61360470917B</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>84fdce5107</t>
+          <t>7a22fe6bd5</t>
         </is>
       </c>
     </row>
@@ -1854,37 +1854,37 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voice AI | Audio Data</t>
+          <t>Data Science Instructor</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>upGrad</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Worldwide</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>himalayas</t>
+          <t>adzuna</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ai, worldwide (place)</t>
+          <t>data science, hyderabad (place)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Entry-level</t>
+          <t>IT Jobs</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://himalayas.app/companies/telus-digital/jobs/ai-speech-audio-specialist-asr-tts-voice-ai-audio-data</t>
+          <t>https://www.adzuna.in/land/ad/5857168441?se=TqYc8W2h8RGhZ7gcUJZivg&amp;utm_medium=api&amp;utm_source=28154f3f&amp;v=CEB40CB7335D41898800C58388A2B035DF674757</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>bb930fc93f</t>
+          <t>84fdce5107</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Financial Accuracy &amp; Tax Logic Expert (AI Community)</t>
+          <t>AI Speech &amp; Audio Specialist – ASR | TTS | Voic